<commit_message>
bat-syncing repo (personal-workstation parity)
</commit_message>
<xml_diff>
--- a/Data/calibration_tracker_log_only.xlsx
+++ b/Data/calibration_tracker_log_only.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\newwb\Documents\brain\professional\university\LCAS\Vicon (EPSURIS) Main\Public Files\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B15D61F-D0BB-429A-9750-840C49EC24BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E613A2C-CEE6-4BC6-893F-378716AC797E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="713" firstSheet="2" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="713" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="WIP" sheetId="1" state="hidden" r:id="rId1"/>
@@ -21,9 +21,6 @@
     <sheet name="SetData" sheetId="24" r:id="rId6"/>
     <sheet name="Problem Cameras" sheetId="23" r:id="rId7"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId8"/>
-  </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">SetData!$E$1:$P$652</definedName>
   </definedNames>
@@ -480,7 +477,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -502,7 +499,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4761" uniqueCount="244">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4779" uniqueCount="262">
   <si>
     <t>How this workbook works</t>
   </si>
@@ -1973,6 +1970,60 @@
   <si>
     <t>Repeated auto-stop straggler</t>
   </si>
+  <si>
+    <t xml:space="preserve">#1 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#2 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#3 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#4 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#5 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#6 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#7 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#8 </t>
+  </si>
+  <si>
+    <t xml:space="preserve">#9 </t>
+  </si>
+  <si>
+    <t>#10</t>
+  </si>
+  <si>
+    <t>#11</t>
+  </si>
+  <si>
+    <t>#12</t>
+  </si>
+  <si>
+    <t>#13</t>
+  </si>
+  <si>
+    <t>#14</t>
+  </si>
+  <si>
+    <t>#15</t>
+  </si>
+  <si>
+    <t>#16</t>
+  </si>
+  <si>
+    <t>#17</t>
+  </si>
+  <si>
+    <t>#18</t>
+  </si>
 </sst>
 </file>
 
@@ -2692,7 +2743,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="154">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -2999,98 +3050,13 @@
     <xf numFmtId="0" fontId="49" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="15" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3100,9 +3066,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="1" fontId="4" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3134,11 +3097,98 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="51" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="17" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="17">
     <dxf>
       <fill>
         <patternFill>
@@ -3292,69 +3342,6 @@
           <bgColor rgb="FFFF9797"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC5D9F1"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFCCCC"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFDE9D9"/>
-        </patternFill>
-      </fill>
-      <border>
-        <left style="thin">
-          <color auto="1"/>
-        </left>
-        <right style="thin">
-          <color auto="1"/>
-        </right>
-        <top style="thin">
-          <color auto="1"/>
-        </top>
-        <bottom style="thin">
-          <color auto="1"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
@@ -3584,154 +3571,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="WIP"/>
-      <sheetName val="Data-Lists"/>
-      <sheetName val="Legend"/>
-      <sheetName val="Log"/>
-      <sheetName val="Daily IE"/>
-      <sheetName val="Daily WE"/>
-      <sheetName val="Errors"/>
-      <sheetName val="Trials"/>
-      <sheetName val="Visualisations"/>
-      <sheetName val="Daily Camera Trends"/>
-      <sheetName val="Daily Averages"/>
-      <sheetName val="Daily Rank"/>
-      <sheetName val="Daily Error Rates"/>
-      <sheetName val="Problem Cameras"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0" refreshError="1"/>
-      <sheetData sheetId="1">
-        <row r="4">
-          <cell r="A4" t="str">
-            <v>#1 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="5">
-          <cell r="A5" t="str">
-            <v>#2 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="6">
-          <cell r="A6" t="str">
-            <v>#3 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="7">
-          <cell r="A7" t="str">
-            <v>#4 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="8">
-          <cell r="A8" t="str">
-            <v>#5 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="9">
-          <cell r="A9" t="str">
-            <v>#6 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="10">
-          <cell r="A10" t="str">
-            <v>#7 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="11">
-          <cell r="A11" t="str">
-            <v>#8 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="12">
-          <cell r="A12" t="str">
-            <v>#9 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="13">
-          <cell r="A13" t="str">
-            <v>#10 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="14">
-          <cell r="A14" t="str">
-            <v>#11 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="15">
-          <cell r="A15" t="str">
-            <v>#12 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="16">
-          <cell r="A16" t="str">
-            <v>#13 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="17">
-          <cell r="A17" t="str">
-            <v>#14 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="18">
-          <cell r="A18" t="str">
-            <v>#15 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="19">
-          <cell r="A19" t="str">
-            <v>#16 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="20">
-          <cell r="A20" t="str">
-            <v>#17 (Vero v2.2)</v>
-          </cell>
-        </row>
-        <row r="21">
-          <cell r="A21" t="str">
-            <v>#18 (Vero v2.2)</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3">
-        <row r="1">
-          <cell r="A1" t="str">
-            <v>DO NOT USE THIS SPREADSHEET, IT IS DEPRECATED AND KEPT ONLY AS REFERENCE FOR FINAL DATA REPRESENTATIONS</v>
-          </cell>
-        </row>
-      </sheetData>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A11174E4-10B8-4B30-8B2E-2E9A5AE08333}" name="CalibrationLog3" displayName="CalibrationLog3" ref="C2:G549" totalsRowShown="0" headerRowDxfId="19" dataDxfId="18">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{A11174E4-10B8-4B30-8B2E-2E9A5AE08333}" name="CalibrationLog3" displayName="CalibrationLog3" ref="C2:G549" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
   <autoFilter ref="C2:G549" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{51B67423-B1B1-4A16-BBCC-834944FAE191}" name="Date" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{FABEBB3C-66EB-4956-95C9-CBB40C9E32E4}" name="Camera" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{766E62E6-E8D6-460F-BDF5-449F20A2F47C}" name="Frame Count" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{132E3B4C-B94B-4FD9-BB91-C8476EF47049}" name="World Error" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{9AE105E3-C1BC-4C8A-A3F2-7EACB47F9196}" name="Image Error" dataDxfId="13"/>
+    <tableColumn id="1" xr3:uid="{51B67423-B1B1-4A16-BBCC-834944FAE191}" name="Date" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{FABEBB3C-66EB-4956-95C9-CBB40C9E32E4}" name="Camera" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{766E62E6-E8D6-460F-BDF5-449F20A2F47C}" name="Frame Count" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{132E3B4C-B94B-4FD9-BB91-C8476EF47049}" name="World Error" dataDxfId="11"/>
+    <tableColumn id="5" xr3:uid="{9AE105E3-C1BC-4C8A-A3F2-7EACB47F9196}" name="Image Error" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -4065,22 +3913,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="130" t="s">
         <v>142</v>
       </c>
-      <c r="B1" s="109"/>
-      <c r="C1" s="109"/>
-      <c r="D1" s="109"/>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
-      <c r="G1" s="109"/>
-      <c r="H1" s="109"/>
-      <c r="I1" s="109"/>
-      <c r="J1" s="109"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="109"/>
-      <c r="M1" s="109"/>
-      <c r="N1" s="109"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="131"/>
+      <c r="L1" s="131"/>
+      <c r="M1" s="131"/>
+      <c r="N1" s="131"/>
     </row>
     <row r="2" spans="1:14" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A2" s="43" t="s">
@@ -4660,26 +4508,26 @@
     <col min="18" max="16384" width="8.88671875" style="70" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="120" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="117" t="s">
+    <row r="1" spans="1:17" s="137" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="134" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="118"/>
-      <c r="C1" s="118"/>
-      <c r="D1" s="118"/>
-      <c r="E1" s="118"/>
-      <c r="F1" s="118"/>
-      <c r="G1" s="118"/>
-      <c r="H1" s="118"/>
-      <c r="I1" s="118"/>
-      <c r="J1" s="118"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="118"/>
-      <c r="M1" s="118"/>
-      <c r="N1" s="118"/>
-      <c r="O1" s="118"/>
-      <c r="P1" s="118"/>
-      <c r="Q1" s="119"/>
+      <c r="B1" s="135"/>
+      <c r="C1" s="135"/>
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="135"/>
+      <c r="G1" s="135"/>
+      <c r="H1" s="135"/>
+      <c r="I1" s="135"/>
+      <c r="J1" s="135"/>
+      <c r="K1" s="135"/>
+      <c r="L1" s="135"/>
+      <c r="M1" s="135"/>
+      <c r="N1" s="135"/>
+      <c r="O1" s="135"/>
+      <c r="P1" s="135"/>
+      <c r="Q1" s="136"/>
     </row>
     <row r="2" spans="1:17" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="8"/>
@@ -4701,12 +4549,12 @@
     </row>
     <row r="3" spans="1:17" customFormat="1" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="8"/>
-      <c r="B3" s="121" t="s">
+      <c r="B3" s="138" t="s">
         <v>182</v>
       </c>
-      <c r="C3" s="122"/>
-      <c r="D3" s="122"/>
-      <c r="E3" s="122"/>
+      <c r="C3" s="139"/>
+      <c r="D3" s="139"/>
+      <c r="E3" s="139"/>
       <c r="F3" s="67"/>
       <c r="G3" s="9"/>
       <c r="H3" s="9"/>
@@ -4734,10 +4582,10 @@
         <v>35</v>
       </c>
       <c r="F4" s="68"/>
-      <c r="G4" s="123" t="s">
+      <c r="G4" s="140" t="s">
         <v>67</v>
       </c>
-      <c r="H4" s="123"/>
+      <c r="H4" s="140"/>
       <c r="I4" s="70"/>
       <c r="J4" s="70"/>
       <c r="K4" s="69"/>
@@ -4764,11 +4612,11 @@
       </c>
       <c r="F5" s="67"/>
       <c r="G5" s="65"/>
-      <c r="H5" s="111" t="s">
+      <c r="H5" s="141" t="s">
         <v>96</v>
       </c>
-      <c r="I5" s="112"/>
-      <c r="J5" s="113"/>
+      <c r="I5" s="142"/>
+      <c r="J5" s="143"/>
       <c r="K5" s="69"/>
       <c r="L5" s="69"/>
       <c r="M5" s="69"/>
@@ -4793,11 +4641,11 @@
       </c>
       <c r="F6" s="67"/>
       <c r="G6" s="66"/>
-      <c r="H6" s="111" t="s">
+      <c r="H6" s="141" t="s">
         <v>95</v>
       </c>
-      <c r="I6" s="112"/>
-      <c r="J6" s="113"/>
+      <c r="I6" s="142"/>
+      <c r="J6" s="143"/>
       <c r="K6" s="69"/>
       <c r="L6" s="69"/>
       <c r="M6" s="69"/>
@@ -4822,11 +4670,11 @@
       </c>
       <c r="F7" s="67"/>
       <c r="G7" s="54"/>
-      <c r="H7" s="111" t="s">
+      <c r="H7" s="141" t="s">
         <v>66</v>
       </c>
-      <c r="I7" s="112"/>
-      <c r="J7" s="113"/>
+      <c r="I7" s="142"/>
+      <c r="J7" s="143"/>
       <c r="K7" s="69"/>
       <c r="L7" s="69"/>
       <c r="M7" s="69"/>
@@ -4877,14 +4725,14 @@
         <v>Yes</v>
       </c>
       <c r="F9" s="67"/>
-      <c r="G9" s="114" t="s">
+      <c r="G9" s="144" t="s">
         <v>178</v>
       </c>
-      <c r="H9" s="115"/>
-      <c r="I9" s="115"/>
-      <c r="J9" s="115"/>
-      <c r="K9" s="115"/>
-      <c r="L9" s="115"/>
+      <c r="H9" s="145"/>
+      <c r="I9" s="145"/>
+      <c r="J9" s="145"/>
+      <c r="K9" s="145"/>
+      <c r="L9" s="145"/>
       <c r="M9" s="69"/>
       <c r="N9" s="8"/>
       <c r="O9" s="8"/>
@@ -4909,15 +4757,15 @@
       <c r="G10" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="116" t="s">
+      <c r="H10" s="146" t="s">
         <v>214</v>
       </c>
-      <c r="I10" s="116"/>
-      <c r="J10" s="116"/>
-      <c r="K10" s="116"/>
-      <c r="L10" s="116"/>
-      <c r="M10" s="116"/>
-      <c r="N10" s="116"/>
+      <c r="I10" s="146"/>
+      <c r="J10" s="146"/>
+      <c r="K10" s="146"/>
+      <c r="L10" s="146"/>
+      <c r="M10" s="146"/>
+      <c r="N10" s="146"/>
       <c r="O10" s="8"/>
       <c r="P10" s="8"/>
     </row>
@@ -4940,15 +4788,15 @@
       <c r="G11" s="29" t="s">
         <v>52</v>
       </c>
-      <c r="H11" s="116" t="s">
+      <c r="H11" s="146" t="s">
         <v>82</v>
       </c>
-      <c r="I11" s="116"/>
-      <c r="J11" s="116"/>
-      <c r="K11" s="116"/>
-      <c r="L11" s="116"/>
-      <c r="M11" s="116"/>
-      <c r="N11" s="116"/>
+      <c r="I11" s="146"/>
+      <c r="J11" s="146"/>
+      <c r="K11" s="146"/>
+      <c r="L11" s="146"/>
+      <c r="M11" s="146"/>
+      <c r="N11" s="146"/>
       <c r="O11" s="8"/>
       <c r="P11" s="8"/>
     </row>
@@ -4971,15 +4819,15 @@
       <c r="G12" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="H12" s="116" t="s">
+      <c r="H12" s="146" t="s">
         <v>149</v>
       </c>
-      <c r="I12" s="116"/>
-      <c r="J12" s="116"/>
-      <c r="K12" s="116"/>
-      <c r="L12" s="116"/>
-      <c r="M12" s="116"/>
-      <c r="N12" s="116"/>
+      <c r="I12" s="146"/>
+      <c r="J12" s="146"/>
+      <c r="K12" s="146"/>
+      <c r="L12" s="146"/>
+      <c r="M12" s="146"/>
+      <c r="N12" s="146"/>
       <c r="O12" s="8"/>
       <c r="P12" s="8"/>
     </row>
@@ -5002,15 +4850,15 @@
       <c r="G13" s="29" t="s">
         <v>112</v>
       </c>
-      <c r="H13" s="116" t="s">
+      <c r="H13" s="146" t="s">
         <v>114</v>
       </c>
-      <c r="I13" s="116"/>
-      <c r="J13" s="116"/>
-      <c r="K13" s="116"/>
-      <c r="L13" s="116"/>
-      <c r="M13" s="116"/>
-      <c r="N13" s="116"/>
+      <c r="I13" s="146"/>
+      <c r="J13" s="146"/>
+      <c r="K13" s="146"/>
+      <c r="L13" s="146"/>
+      <c r="M13" s="146"/>
+      <c r="N13" s="146"/>
       <c r="O13" s="8"/>
       <c r="P13" s="8"/>
     </row>
@@ -5033,15 +4881,15 @@
       <c r="G14" s="29" t="s">
         <v>113</v>
       </c>
-      <c r="H14" s="116" t="s">
+      <c r="H14" s="146" t="s">
         <v>147</v>
       </c>
-      <c r="I14" s="116"/>
-      <c r="J14" s="116"/>
-      <c r="K14" s="116"/>
-      <c r="L14" s="116"/>
-      <c r="M14" s="116"/>
-      <c r="N14" s="116"/>
+      <c r="I14" s="146"/>
+      <c r="J14" s="146"/>
+      <c r="K14" s="146"/>
+      <c r="L14" s="146"/>
+      <c r="M14" s="146"/>
+      <c r="N14" s="146"/>
       <c r="O14" s="8"/>
       <c r="P14" s="8"/>
     </row>
@@ -5064,15 +4912,15 @@
       <c r="G15" s="29" t="s">
         <v>115</v>
       </c>
-      <c r="H15" s="116" t="s">
+      <c r="H15" s="146" t="s">
         <v>117</v>
       </c>
-      <c r="I15" s="116"/>
-      <c r="J15" s="116"/>
-      <c r="K15" s="116"/>
-      <c r="L15" s="116"/>
-      <c r="M15" s="116"/>
-      <c r="N15" s="116"/>
+      <c r="I15" s="146"/>
+      <c r="J15" s="146"/>
+      <c r="K15" s="146"/>
+      <c r="L15" s="146"/>
+      <c r="M15" s="146"/>
+      <c r="N15" s="146"/>
       <c r="O15" s="8"/>
       <c r="P15" s="8"/>
     </row>
@@ -5095,15 +4943,15 @@
       <c r="G16" s="29" t="s">
         <v>116</v>
       </c>
-      <c r="H16" s="116" t="s">
+      <c r="H16" s="146" t="s">
         <v>148</v>
       </c>
-      <c r="I16" s="116"/>
-      <c r="J16" s="116"/>
-      <c r="K16" s="116"/>
-      <c r="L16" s="116"/>
-      <c r="M16" s="116"/>
-      <c r="N16" s="116"/>
+      <c r="I16" s="146"/>
+      <c r="J16" s="146"/>
+      <c r="K16" s="146"/>
+      <c r="L16" s="146"/>
+      <c r="M16" s="146"/>
+      <c r="N16" s="146"/>
       <c r="O16" s="8"/>
       <c r="P16" s="8"/>
     </row>
@@ -5126,15 +4974,15 @@
       <c r="G17" s="71" t="s">
         <v>176</v>
       </c>
-      <c r="H17" s="110" t="s">
+      <c r="H17" s="133" t="s">
         <v>184</v>
       </c>
-      <c r="I17" s="110"/>
-      <c r="J17" s="110"/>
-      <c r="K17" s="110"/>
-      <c r="L17" s="110"/>
-      <c r="M17" s="110"/>
-      <c r="N17" s="110"/>
+      <c r="I17" s="133"/>
+      <c r="J17" s="133"/>
+      <c r="K17" s="133"/>
+      <c r="L17" s="133"/>
+      <c r="M17" s="133"/>
+      <c r="N17" s="133"/>
       <c r="O17" s="8"/>
       <c r="P17" s="8"/>
     </row>
@@ -5157,15 +5005,15 @@
       <c r="G18" s="71" t="s">
         <v>185</v>
       </c>
-      <c r="H18" s="110" t="s">
+      <c r="H18" s="133" t="s">
         <v>195</v>
       </c>
-      <c r="I18" s="110"/>
-      <c r="J18" s="110"/>
-      <c r="K18" s="110"/>
-      <c r="L18" s="110"/>
-      <c r="M18" s="110"/>
-      <c r="N18" s="110"/>
+      <c r="I18" s="133"/>
+      <c r="J18" s="133"/>
+      <c r="K18" s="133"/>
+      <c r="L18" s="133"/>
+      <c r="M18" s="133"/>
+      <c r="N18" s="133"/>
       <c r="O18" s="8"/>
       <c r="P18" s="8"/>
     </row>
@@ -5188,15 +5036,15 @@
       <c r="G19" s="71" t="s">
         <v>64</v>
       </c>
-      <c r="H19" s="135" t="s">
+      <c r="H19" s="132" t="s">
         <v>236</v>
       </c>
-      <c r="I19" s="110"/>
-      <c r="J19" s="110"/>
-      <c r="K19" s="110"/>
-      <c r="L19" s="110"/>
-      <c r="M19" s="110"/>
-      <c r="N19" s="110"/>
+      <c r="I19" s="133"/>
+      <c r="J19" s="133"/>
+      <c r="K19" s="133"/>
+      <c r="L19" s="133"/>
+      <c r="M19" s="133"/>
+      <c r="N19" s="133"/>
       <c r="O19" s="8"/>
       <c r="P19" s="8"/>
     </row>
@@ -5320,6 +5168,7 @@
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="17">
+    <mergeCell ref="H12:N12"/>
     <mergeCell ref="H19:N19"/>
     <mergeCell ref="A1:XFD1"/>
     <mergeCell ref="B3:E3"/>
@@ -5336,7 +5185,6 @@
     <mergeCell ref="H14:N14"/>
     <mergeCell ref="H10:N10"/>
     <mergeCell ref="H11:N11"/>
-    <mergeCell ref="H12:N12"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:E22">
     <cfRule type="expression" dxfId="9" priority="1">
@@ -5352,7 +5200,7 @@
   <sheetPr>
     <tabColor theme="3" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:O3116"/>
+  <dimension ref="A1:M3116"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.77734375" style="38" customWidth="1"/>
@@ -5364,20 +5212,20 @@
     <col min="7" max="7" width="17.44140625" style="33" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="124" t="s">
+    <row r="1" spans="1:13" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="147" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="125"/>
-      <c r="C1" s="125"/>
-      <c r="D1" s="125"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="127" t="s">
+      <c r="B1" s="148"/>
+      <c r="C1" s="148"/>
+      <c r="D1" s="148"/>
+      <c r="E1" s="149"/>
+      <c r="F1" s="150" t="s">
         <v>65</v>
       </c>
-      <c r="G1" s="127"/>
-    </row>
-    <row r="2" spans="1:15" s="31" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G1" s="150"/>
+    </row>
+    <row r="2" spans="1:13" s="31" customFormat="1" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="47" t="s">
         <v>61</v>
       </c>
@@ -5393,14 +5241,14 @@
       <c r="E2" s="64" t="s">
         <v>167</v>
       </c>
-      <c r="F2" s="140" t="s">
+      <c r="F2" s="111" t="s">
         <v>32</v>
       </c>
       <c r="G2" s="41" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" s="34" t="s">
         <v>57</v>
       </c>
@@ -5419,11 +5267,11 @@
       <c r="F3" s="37">
         <v>0.274982</v>
       </c>
-      <c r="G3" s="141">
+      <c r="G3" s="112">
         <v>7.9356800000000005E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" s="34" t="s">
         <v>57</v>
       </c>
@@ -5442,11 +5290,11 @@
       <c r="F4" s="37">
         <v>0.42184300000000002</v>
       </c>
-      <c r="G4" s="141">
+      <c r="G4" s="112">
         <v>0.112306</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" s="34" t="s">
         <v>57</v>
       </c>
@@ -5465,19 +5313,11 @@
       <c r="F5" s="37">
         <v>0.39858399999999999</v>
       </c>
-      <c r="G5" s="141">
+      <c r="G5" s="112">
         <v>9.2427499999999996E-2</v>
       </c>
-      <c r="H5" s="136"/>
-      <c r="I5" s="136"/>
-      <c r="J5" s="136"/>
-      <c r="K5" s="136"/>
-      <c r="L5" s="136"/>
-      <c r="M5" s="136"/>
-      <c r="N5" s="136"/>
-      <c r="O5" s="136"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" s="34" t="s">
         <v>57</v>
       </c>
@@ -5496,19 +5336,11 @@
       <c r="F6" s="37">
         <v>0.62003600000000003</v>
       </c>
-      <c r="G6" s="141">
+      <c r="G6" s="112">
         <v>0.12157900000000001</v>
       </c>
-      <c r="H6" s="136"/>
-      <c r="I6" s="136"/>
-      <c r="J6" s="136"/>
-      <c r="K6" s="136"/>
-      <c r="L6" s="136"/>
-      <c r="M6" s="136"/>
-      <c r="N6" s="136"/>
-      <c r="O6" s="136"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" s="34" t="s">
         <v>57</v>
       </c>
@@ -5527,19 +5359,17 @@
       <c r="F7" s="37">
         <v>0.19189300000000001</v>
       </c>
-      <c r="G7" s="141">
+      <c r="G7" s="112">
         <v>4.4366900000000001E-2</v>
       </c>
-      <c r="H7" s="137"/>
-      <c r="I7" s="137"/>
-      <c r="J7" s="137"/>
-      <c r="K7" s="137"/>
-      <c r="L7" s="137"/>
-      <c r="M7" s="137"/>
-      <c r="N7" s="136"/>
-      <c r="O7" s="136"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H7" s="108"/>
+      <c r="I7" s="108"/>
+      <c r="J7" s="108"/>
+      <c r="K7" s="108"/>
+      <c r="L7" s="108"/>
+      <c r="M7" s="108"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" s="34" t="s">
         <v>57</v>
       </c>
@@ -5558,19 +5388,17 @@
       <c r="F8" s="37">
         <v>0.44223499999999999</v>
       </c>
-      <c r="G8" s="141">
+      <c r="G8" s="112">
         <v>8.9975399999999997E-2</v>
       </c>
-      <c r="H8" s="137"/>
-      <c r="I8" s="137"/>
-      <c r="J8" s="137"/>
-      <c r="K8" s="137"/>
-      <c r="L8" s="137"/>
-      <c r="M8" s="137"/>
-      <c r="N8" s="136"/>
-      <c r="O8" s="136"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H8" s="108"/>
+      <c r="I8" s="108"/>
+      <c r="J8" s="108"/>
+      <c r="K8" s="108"/>
+      <c r="L8" s="108"/>
+      <c r="M8" s="108"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" s="34" t="s">
         <v>57</v>
       </c>
@@ -5589,19 +5417,17 @@
       <c r="F9" s="37">
         <v>0.50989600000000002</v>
       </c>
-      <c r="G9" s="141">
+      <c r="G9" s="112">
         <v>0.102799</v>
       </c>
-      <c r="H9" s="137"/>
-      <c r="I9" s="137"/>
-      <c r="J9" s="137"/>
-      <c r="K9" s="137"/>
-      <c r="L9" s="137"/>
-      <c r="M9" s="137"/>
-      <c r="N9" s="136"/>
-      <c r="O9" s="136"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H9" s="108"/>
+      <c r="I9" s="108"/>
+      <c r="J9" s="108"/>
+      <c r="K9" s="108"/>
+      <c r="L9" s="108"/>
+      <c r="M9" s="108"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" s="34" t="s">
         <v>57</v>
       </c>
@@ -5620,19 +5446,17 @@
       <c r="F10" s="37">
         <v>0.39593499999999998</v>
       </c>
-      <c r="G10" s="141">
+      <c r="G10" s="112">
         <v>7.95796E-2</v>
       </c>
-      <c r="H10" s="137"/>
-      <c r="I10" s="137"/>
-      <c r="J10" s="137"/>
-      <c r="K10" s="137"/>
-      <c r="L10" s="137"/>
-      <c r="M10" s="137"/>
-      <c r="N10" s="136"/>
-      <c r="O10" s="136"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H10" s="108"/>
+      <c r="I10" s="108"/>
+      <c r="J10" s="108"/>
+      <c r="K10" s="108"/>
+      <c r="L10" s="108"/>
+      <c r="M10" s="108"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" s="34" t="s">
         <v>57</v>
       </c>
@@ -5651,19 +5475,17 @@
       <c r="F11" s="37">
         <v>0.49960599999999999</v>
       </c>
-      <c r="G11" s="141">
+      <c r="G11" s="112">
         <v>0.13203699999999999</v>
       </c>
-      <c r="H11" s="137"/>
-      <c r="I11" s="137"/>
-      <c r="J11" s="137"/>
-      <c r="K11" s="137"/>
-      <c r="L11" s="137"/>
-      <c r="M11" s="137"/>
-      <c r="N11" s="136"/>
-      <c r="O11" s="136"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H11" s="108"/>
+      <c r="I11" s="108"/>
+      <c r="J11" s="108"/>
+      <c r="K11" s="108"/>
+      <c r="L11" s="108"/>
+      <c r="M11" s="108"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" s="34" t="s">
         <v>57</v>
       </c>
@@ -5682,19 +5504,17 @@
       <c r="F12" s="37">
         <v>0.13059299999999999</v>
       </c>
-      <c r="G12" s="141">
+      <c r="G12" s="112">
         <v>4.5056100000000002E-2</v>
       </c>
-      <c r="H12" s="137"/>
-      <c r="I12" s="137"/>
-      <c r="J12" s="137"/>
-      <c r="K12" s="137"/>
-      <c r="L12" s="137"/>
-      <c r="M12" s="137"/>
-      <c r="N12" s="136"/>
-      <c r="O12" s="136"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H12" s="108"/>
+      <c r="I12" s="108"/>
+      <c r="J12" s="108"/>
+      <c r="K12" s="108"/>
+      <c r="L12" s="108"/>
+      <c r="M12" s="108"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" s="34" t="s">
         <v>57</v>
       </c>
@@ -5713,19 +5533,17 @@
       <c r="F13" s="37">
         <v>0.428371</v>
       </c>
-      <c r="G13" s="141">
+      <c r="G13" s="112">
         <v>0.14066300000000001</v>
       </c>
-      <c r="H13" s="137"/>
-      <c r="I13" s="137"/>
-      <c r="J13" s="137"/>
-      <c r="K13" s="137"/>
-      <c r="L13" s="137"/>
-      <c r="M13" s="137"/>
-      <c r="N13" s="136"/>
-      <c r="O13" s="136"/>
-    </row>
-    <row r="14" spans="1:15" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H13" s="108"/>
+      <c r="I13" s="108"/>
+      <c r="J13" s="108"/>
+      <c r="K13" s="108"/>
+      <c r="L13" s="108"/>
+      <c r="M13" s="108"/>
+    </row>
+    <row r="14" spans="1:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="34" t="s">
         <v>57</v>
       </c>
@@ -5744,19 +5562,17 @@
       <c r="F14" s="37">
         <v>0.16838600000000001</v>
       </c>
-      <c r="G14" s="141">
+      <c r="G14" s="112">
         <v>4.2415799999999997E-2</v>
       </c>
-      <c r="H14" s="138"/>
-      <c r="I14" s="138"/>
-      <c r="J14" s="138"/>
-      <c r="K14" s="138"/>
-      <c r="L14" s="138"/>
-      <c r="M14" s="138"/>
-      <c r="N14" s="136"/>
-      <c r="O14" s="136"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H14" s="109"/>
+      <c r="I14" s="109"/>
+      <c r="J14" s="109"/>
+      <c r="K14" s="109"/>
+      <c r="L14" s="109"/>
+      <c r="M14" s="109"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" s="34" t="s">
         <v>57</v>
       </c>
@@ -5775,19 +5591,17 @@
       <c r="F15" s="37">
         <v>0.160743</v>
       </c>
-      <c r="G15" s="141">
+      <c r="G15" s="112">
         <v>4.9050299999999998E-2</v>
       </c>
-      <c r="H15" s="138"/>
-      <c r="I15" s="138"/>
-      <c r="J15" s="138"/>
-      <c r="K15" s="138"/>
-      <c r="L15" s="138"/>
-      <c r="M15" s="138"/>
-      <c r="N15" s="136"/>
-      <c r="O15" s="136"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H15" s="109"/>
+      <c r="I15" s="109"/>
+      <c r="J15" s="109"/>
+      <c r="K15" s="109"/>
+      <c r="L15" s="109"/>
+      <c r="M15" s="109"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" s="34" t="s">
         <v>57</v>
       </c>
@@ -5806,19 +5620,11 @@
       <c r="F16" s="37">
         <v>0.43960500000000002</v>
       </c>
-      <c r="G16" s="141">
+      <c r="G16" s="112">
         <v>0.10267900000000001</v>
       </c>
-      <c r="H16" s="136"/>
-      <c r="I16" s="136"/>
-      <c r="J16" s="136"/>
-      <c r="K16" s="136"/>
-      <c r="L16" s="136"/>
-      <c r="M16" s="136"/>
-      <c r="N16" s="136"/>
-      <c r="O16" s="136"/>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="34" t="s">
         <v>57</v>
       </c>
@@ -5837,19 +5643,11 @@
       <c r="F17" s="37">
         <v>0.64795899999999995</v>
       </c>
-      <c r="G17" s="141">
+      <c r="G17" s="112">
         <v>0.147318</v>
       </c>
-      <c r="H17" s="136"/>
-      <c r="I17" s="136"/>
-      <c r="J17" s="136"/>
-      <c r="K17" s="136"/>
-      <c r="L17" s="136"/>
-      <c r="M17" s="136"/>
-      <c r="N17" s="136"/>
-      <c r="O17" s="136"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="34" t="s">
         <v>57</v>
       </c>
@@ -5868,19 +5666,14 @@
       <c r="F18" s="37">
         <v>0.37152299999999999</v>
       </c>
-      <c r="G18" s="141">
+      <c r="G18" s="112">
         <v>7.7194100000000002E-2</v>
       </c>
-      <c r="H18" s="139"/>
-      <c r="I18" s="139"/>
-      <c r="J18" s="139"/>
-      <c r="K18" s="136"/>
-      <c r="L18" s="136"/>
-      <c r="M18" s="136"/>
-      <c r="N18" s="136"/>
-      <c r="O18" s="136"/>
-    </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H18" s="110"/>
+      <c r="I18" s="110"/>
+      <c r="J18" s="110"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="34" t="s">
         <v>57</v>
       </c>
@@ -5899,19 +5692,14 @@
       <c r="F19" s="37">
         <v>0.54793400000000003</v>
       </c>
-      <c r="G19" s="141">
+      <c r="G19" s="112">
         <v>0.109931</v>
       </c>
-      <c r="H19" s="139"/>
-      <c r="I19" s="139"/>
-      <c r="J19" s="139"/>
-      <c r="K19" s="136"/>
-      <c r="L19" s="136"/>
-      <c r="M19" s="136"/>
-      <c r="N19" s="136"/>
-      <c r="O19" s="136"/>
-    </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="H19" s="110"/>
+      <c r="I19" s="110"/>
+      <c r="J19" s="110"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="34" t="s">
         <v>57</v>
       </c>
@@ -5930,19 +5718,11 @@
       <c r="F20" s="37">
         <v>0.38631799999999999</v>
       </c>
-      <c r="G20" s="141">
+      <c r="G20" s="112">
         <v>0.10861</v>
       </c>
-      <c r="H20" s="136"/>
-      <c r="I20" s="136"/>
-      <c r="J20" s="136"/>
-      <c r="K20" s="136"/>
-      <c r="L20" s="136"/>
-      <c r="M20" s="136"/>
-      <c r="N20" s="136"/>
-      <c r="O20" s="136"/>
-    </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="34" t="s">
         <v>57</v>
       </c>
@@ -5961,19 +5741,11 @@
       <c r="F21" s="37">
         <v>0.40509299999999998</v>
       </c>
-      <c r="G21" s="141">
+      <c r="G21" s="112">
         <v>0.10678</v>
       </c>
-      <c r="H21" s="136"/>
-      <c r="I21" s="136"/>
-      <c r="J21" s="136"/>
-      <c r="K21" s="136"/>
-      <c r="L21" s="136"/>
-      <c r="M21" s="136"/>
-      <c r="N21" s="136"/>
-      <c r="O21" s="136"/>
-    </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="34" t="s">
         <v>57</v>
       </c>
@@ -5992,19 +5764,11 @@
       <c r="F22" s="37">
         <v>0.42063299999999998</v>
       </c>
-      <c r="G22" s="141">
+      <c r="G22" s="112">
         <v>9.8741200000000001E-2</v>
       </c>
-      <c r="H22" s="136"/>
-      <c r="I22" s="136"/>
-      <c r="J22" s="136"/>
-      <c r="K22" s="136"/>
-      <c r="L22" s="136"/>
-      <c r="M22" s="136"/>
-      <c r="N22" s="136"/>
-      <c r="O22" s="136"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="34" t="s">
         <v>57</v>
       </c>
@@ -6023,19 +5787,11 @@
       <c r="F23" s="37">
         <v>0.610344</v>
       </c>
-      <c r="G23" s="141">
+      <c r="G23" s="112">
         <v>0.120907</v>
       </c>
-      <c r="H23" s="136"/>
-      <c r="I23" s="136"/>
-      <c r="J23" s="136"/>
-      <c r="K23" s="136"/>
-      <c r="L23" s="136"/>
-      <c r="M23" s="136"/>
-      <c r="N23" s="136"/>
-      <c r="O23" s="136"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="34" t="s">
         <v>57</v>
       </c>
@@ -6054,11 +5810,11 @@
       <c r="F24" s="37">
         <v>0.28196100000000002</v>
       </c>
-      <c r="G24" s="141">
+      <c r="G24" s="112">
         <v>6.7092299999999994E-2</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="34" t="s">
         <v>57</v>
       </c>
@@ -6077,11 +5833,11 @@
       <c r="F25" s="37">
         <v>0.35003099999999998</v>
       </c>
-      <c r="G25" s="141">
+      <c r="G25" s="112">
         <v>7.3608499999999993E-2</v>
       </c>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="34" t="s">
         <v>57</v>
       </c>
@@ -6100,11 +5856,11 @@
       <c r="F26" s="37">
         <v>0.36660399999999999</v>
       </c>
-      <c r="G26" s="141">
+      <c r="G26" s="112">
         <v>7.6716000000000006E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="34" t="s">
         <v>57</v>
       </c>
@@ -6123,11 +5879,11 @@
       <c r="F27" s="37">
         <v>0.162101</v>
       </c>
-      <c r="G27" s="141">
+      <c r="G27" s="112">
         <v>4.9118500000000002E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="34" t="s">
         <v>57</v>
       </c>
@@ -6146,11 +5902,11 @@
       <c r="F28" s="37">
         <v>0.42067700000000002</v>
       </c>
-      <c r="G28" s="141">
+      <c r="G28" s="112">
         <v>8.1860199999999994E-2</v>
       </c>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="34" t="s">
         <v>57</v>
       </c>
@@ -6169,11 +5925,11 @@
       <c r="F29" s="37">
         <v>0.45557700000000001</v>
       </c>
-      <c r="G29" s="141">
+      <c r="G29" s="112">
         <v>0.123795</v>
       </c>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="34" t="s">
         <v>57</v>
       </c>
@@ -6192,11 +5948,11 @@
       <c r="F30" s="37">
         <v>0.43718499999999999</v>
       </c>
-      <c r="G30" s="141">
+      <c r="G30" s="112">
         <v>0.14344199999999999</v>
       </c>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="34" t="s">
         <v>57</v>
       </c>
@@ -6215,11 +5971,11 @@
       <c r="F31" s="37">
         <v>0.30209799999999998</v>
       </c>
-      <c r="G31" s="141">
+      <c r="G31" s="112">
         <v>9.3080999999999997E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="34" t="s">
         <v>57</v>
       </c>
@@ -6238,7 +5994,7 @@
       <c r="F32" s="37">
         <v>0.18565499999999999</v>
       </c>
-      <c r="G32" s="141">
+      <c r="G32" s="112">
         <v>4.46854E-2</v>
       </c>
     </row>
@@ -6261,7 +6017,7 @@
       <c r="F33" s="37">
         <v>0.21656300000000001</v>
       </c>
-      <c r="G33" s="141">
+      <c r="G33" s="112">
         <v>6.9651900000000003E-2</v>
       </c>
     </row>
@@ -6284,7 +6040,7 @@
       <c r="F34" s="37">
         <v>0.46116299999999999</v>
       </c>
-      <c r="G34" s="141">
+      <c r="G34" s="112">
         <v>0.104768</v>
       </c>
     </row>
@@ -6307,7 +6063,7 @@
       <c r="F35" s="37">
         <v>0.49668299999999999</v>
       </c>
-      <c r="G35" s="141">
+      <c r="G35" s="112">
         <v>0.111633</v>
       </c>
     </row>
@@ -6330,7 +6086,7 @@
       <c r="F36" s="37">
         <v>0.32052799999999998</v>
       </c>
-      <c r="G36" s="141">
+      <c r="G36" s="112">
         <v>6.6401399999999999E-2</v>
       </c>
     </row>
@@ -6353,7 +6109,7 @@
       <c r="F37" s="37">
         <v>0.56830499999999995</v>
       </c>
-      <c r="G37" s="141">
+      <c r="G37" s="112">
         <v>0.114508</v>
       </c>
     </row>
@@ -6376,7 +6132,7 @@
       <c r="F38" s="37">
         <v>0.32684800000000003</v>
       </c>
-      <c r="G38" s="141">
+      <c r="G38" s="112">
         <v>9.1957899999999995E-2</v>
       </c>
     </row>
@@ -6399,7 +6155,7 @@
       <c r="F39" s="37">
         <v>0.55680700000000005</v>
       </c>
-      <c r="G39" s="141">
+      <c r="G39" s="112">
         <v>0.14671400000000001</v>
       </c>
     </row>
@@ -6422,7 +6178,7 @@
       <c r="F40" s="37">
         <v>0.34914299999999998</v>
       </c>
-      <c r="G40" s="141">
+      <c r="G40" s="112">
         <v>8.1951999999999997E-2</v>
       </c>
     </row>
@@ -6445,7 +6201,7 @@
       <c r="F41" s="37">
         <v>0.55386500000000005</v>
       </c>
-      <c r="G41" s="141">
+      <c r="G41" s="112">
         <v>0.109685</v>
       </c>
     </row>
@@ -6468,7 +6224,7 @@
       <c r="F42" s="37">
         <v>0.32659700000000003</v>
       </c>
-      <c r="G42" s="141">
+      <c r="G42" s="112">
         <v>7.7769500000000005E-2</v>
       </c>
     </row>
@@ -6491,7 +6247,7 @@
       <c r="F43" s="37">
         <v>0.39977800000000002</v>
       </c>
-      <c r="G43" s="141">
+      <c r="G43" s="112">
         <v>8.4118100000000001E-2</v>
       </c>
     </row>
@@ -6514,7 +6270,7 @@
       <c r="F44" s="37">
         <v>0.42612899999999998</v>
       </c>
-      <c r="G44" s="141">
+      <c r="G44" s="112">
         <v>8.9207099999999998E-2</v>
       </c>
     </row>
@@ -6537,7 +6293,7 @@
       <c r="F45" s="37">
         <v>0.157855</v>
       </c>
-      <c r="G45" s="141">
+      <c r="G45" s="112">
         <v>4.7859600000000002E-2</v>
       </c>
     </row>
@@ -6560,7 +6316,7 @@
       <c r="F46" s="37">
         <v>0.35114800000000002</v>
       </c>
-      <c r="G46" s="141">
+      <c r="G46" s="112">
         <v>6.8267099999999997E-2</v>
       </c>
     </row>
@@ -6583,7 +6339,7 @@
       <c r="F47" s="37">
         <v>0.508247</v>
       </c>
-      <c r="G47" s="141">
+      <c r="G47" s="112">
         <v>0.13811000000000001</v>
       </c>
     </row>
@@ -6606,7 +6362,7 @@
       <c r="F48" s="37">
         <v>0.36122100000000001</v>
       </c>
-      <c r="G48" s="141">
+      <c r="G48" s="112">
         <v>0.118642</v>
       </c>
     </row>
@@ -6629,7 +6385,7 @@
       <c r="F49" s="37">
         <v>0.19215299999999999</v>
       </c>
-      <c r="G49" s="141">
+      <c r="G49" s="112">
         <v>5.9232199999999999E-2</v>
       </c>
     </row>
@@ -6652,7 +6408,7 @@
       <c r="F50" s="37">
         <v>0.220161</v>
       </c>
-      <c r="G50" s="141">
+      <c r="G50" s="112">
         <v>5.2973800000000001E-2</v>
       </c>
     </row>
@@ -6675,7 +6431,7 @@
       <c r="F51" s="37">
         <v>0.19145999999999999</v>
       </c>
-      <c r="G51" s="141">
+      <c r="G51" s="112">
         <v>6.1579000000000002E-2</v>
       </c>
     </row>
@@ -6698,7 +6454,7 @@
       <c r="F52" s="37">
         <v>0.29572300000000001</v>
       </c>
-      <c r="G52" s="141">
+      <c r="G52" s="112">
         <v>6.7059099999999996E-2</v>
       </c>
     </row>
@@ -6721,7 +6477,7 @@
       <c r="F53" s="37">
         <v>0.29070200000000002</v>
       </c>
-      <c r="G53" s="141">
+      <c r="G53" s="112">
         <v>6.5277500000000002E-2</v>
       </c>
     </row>
@@ -6744,7 +6500,7 @@
       <c r="F54" s="37">
         <v>0.33533099999999999</v>
       </c>
-      <c r="G54" s="141">
+      <c r="G54" s="112">
         <v>6.9472199999999998E-2</v>
       </c>
     </row>
@@ -6767,7 +6523,7 @@
       <c r="F55" s="37">
         <v>0.47264099999999998</v>
       </c>
-      <c r="G55" s="141">
+      <c r="G55" s="112">
         <v>9.5271300000000003E-2</v>
       </c>
     </row>
@@ -6790,7 +6546,7 @@
       <c r="F56" s="37">
         <v>0.28613699999999997</v>
       </c>
-      <c r="G56" s="141">
+      <c r="G56" s="112">
         <v>8.0479400000000006E-2</v>
       </c>
     </row>
@@ -6813,7 +6569,7 @@
       <c r="F57" s="37">
         <v>0.39689600000000003</v>
       </c>
-      <c r="G57" s="141">
+      <c r="G57" s="112">
         <v>0.104628</v>
       </c>
     </row>
@@ -6836,7 +6592,7 @@
       <c r="F58" s="37">
         <v>0.45231500000000002</v>
       </c>
-      <c r="G58" s="141">
+      <c r="G58" s="112">
         <v>0.106193</v>
       </c>
     </row>
@@ -6859,7 +6615,7 @@
       <c r="F59" s="37">
         <v>0.56917399999999996</v>
       </c>
-      <c r="G59" s="141">
+      <c r="G59" s="112">
         <v>0.112651</v>
       </c>
     </row>
@@ -6882,7 +6638,7 @@
       <c r="F60" s="37">
         <v>0.27124799999999999</v>
       </c>
-      <c r="G60" s="141">
+      <c r="G60" s="112">
         <v>6.4562400000000006E-2</v>
       </c>
     </row>
@@ -6905,7 +6661,7 @@
       <c r="F61" s="37">
         <v>0.38306699999999999</v>
       </c>
-      <c r="G61" s="141">
+      <c r="G61" s="112">
         <v>8.06085E-2</v>
       </c>
     </row>
@@ -6928,7 +6684,7 @@
       <c r="F62" s="37">
         <v>0.39710200000000001</v>
       </c>
-      <c r="G62" s="141">
+      <c r="G62" s="112">
         <v>8.3112099999999994E-2</v>
       </c>
     </row>
@@ -6951,7 +6707,7 @@
       <c r="F63" s="37">
         <v>0.228356</v>
       </c>
-      <c r="G63" s="141">
+      <c r="G63" s="112">
         <v>6.9231899999999999E-2</v>
       </c>
     </row>
@@ -6974,7 +6730,7 @@
       <c r="F64" s="37">
         <v>0.439106</v>
       </c>
-      <c r="G64" s="141">
+      <c r="G64" s="112">
         <v>8.5488999999999996E-2</v>
       </c>
     </row>
@@ -6997,7 +6753,7 @@
       <c r="F65" s="37">
         <v>0.50203399999999998</v>
       </c>
-      <c r="G65" s="141">
+      <c r="G65" s="112">
         <v>0.136459</v>
       </c>
     </row>
@@ -7020,7 +6776,7 @@
       <c r="F66" s="37">
         <v>0.40054099999999998</v>
       </c>
-      <c r="G66" s="141">
+      <c r="G66" s="112">
         <v>0.13156499999999999</v>
       </c>
     </row>
@@ -7043,7 +6799,7 @@
       <c r="F67" s="37">
         <v>0.20336000000000001</v>
       </c>
-      <c r="G67" s="141">
+      <c r="G67" s="112">
         <v>6.2631199999999998E-2</v>
       </c>
     </row>
@@ -7066,7 +6822,7 @@
       <c r="F68" s="37">
         <v>0.25667299999999998</v>
       </c>
-      <c r="G68" s="141">
+      <c r="G68" s="112">
         <v>6.1802799999999998E-2</v>
       </c>
     </row>
@@ -7089,7 +6845,7 @@
       <c r="F69" s="37">
         <v>0.18460799999999999</v>
       </c>
-      <c r="G69" s="141">
+      <c r="G69" s="112">
         <v>5.9381200000000002E-2</v>
       </c>
     </row>
@@ -7112,7 +6868,7 @@
       <c r="F70" s="37">
         <v>0.437442</v>
       </c>
-      <c r="G70" s="141">
+      <c r="G70" s="112">
         <v>9.9357200000000007E-2</v>
       </c>
     </row>
@@ -7135,7 +6891,7 @@
       <c r="F71" s="37">
         <v>0.355014</v>
       </c>
-      <c r="G71" s="141">
+      <c r="G71" s="112">
         <v>7.9746600000000001E-2</v>
       </c>
     </row>
@@ -7158,7 +6914,7 @@
       <c r="F72" s="37">
         <v>0.354182</v>
       </c>
-      <c r="G72" s="141">
+      <c r="G72" s="112">
         <v>7.3407E-2</v>
       </c>
     </row>
@@ -7181,7 +6937,7 @@
       <c r="F73" s="37">
         <v>0.53930999999999996</v>
       </c>
-      <c r="G73" s="141">
+      <c r="G73" s="112">
         <v>0.10856499999999999</v>
       </c>
     </row>
@@ -7204,7 +6960,7 @@
       <c r="F74" s="37">
         <v>0.21954399999999999</v>
       </c>
-      <c r="G74" s="141">
+      <c r="G74" s="112">
         <v>6.17744E-2</v>
       </c>
     </row>
@@ -7227,7 +6983,7 @@
       <c r="F75" s="37">
         <v>0.37991200000000003</v>
       </c>
-      <c r="G75" s="141">
+      <c r="G75" s="112">
         <v>0.10016</v>
       </c>
     </row>
@@ -7250,7 +7006,7 @@
       <c r="F76" s="37">
         <v>0.43276999999999999</v>
       </c>
-      <c r="G76" s="141">
+      <c r="G76" s="112">
         <v>0.101578</v>
       </c>
     </row>
@@ -7273,7 +7029,7 @@
       <c r="F77" s="37">
         <v>0.45406200000000002</v>
       </c>
-      <c r="G77" s="141">
+      <c r="G77" s="112">
         <v>8.9885099999999996E-2</v>
       </c>
     </row>
@@ -7296,7 +7052,7 @@
       <c r="F78" s="37">
         <v>0.258108</v>
       </c>
-      <c r="G78" s="141">
+      <c r="G78" s="112">
         <v>6.1423999999999999E-2</v>
       </c>
     </row>
@@ -7319,7 +7075,7 @@
       <c r="F79" s="37">
         <v>0.33665899999999999</v>
       </c>
-      <c r="G79" s="141">
+      <c r="G79" s="112">
         <v>7.0834300000000003E-2</v>
       </c>
     </row>
@@ -7342,7 +7098,7 @@
       <c r="F80" s="37">
         <v>0.380859</v>
       </c>
-      <c r="G80" s="141">
+      <c r="G80" s="112">
         <v>7.9699599999999995E-2</v>
       </c>
     </row>
@@ -7365,7 +7121,7 @@
       <c r="F81" s="37">
         <v>0.211755</v>
       </c>
-      <c r="G81" s="141">
+      <c r="G81" s="112">
         <v>6.4197799999999999E-2</v>
       </c>
     </row>
@@ -7388,7 +7144,7 @@
       <c r="F82" s="37">
         <v>0.42335200000000001</v>
       </c>
-      <c r="G82" s="141">
+      <c r="G82" s="112">
         <v>8.2395399999999994E-2</v>
       </c>
     </row>
@@ -7411,7 +7167,7 @@
       <c r="F83" s="37">
         <v>0.26177600000000001</v>
       </c>
-      <c r="G83" s="141">
+      <c r="G83" s="112">
         <v>7.1129800000000007E-2</v>
       </c>
     </row>
@@ -7434,7 +7190,7 @@
       <c r="F84" s="37">
         <v>0.37280799999999997</v>
       </c>
-      <c r="G84" s="141">
+      <c r="G84" s="112">
         <v>0.12241299999999999</v>
       </c>
     </row>
@@ -7457,7 +7213,7 @@
       <c r="F85" s="37">
         <v>0.27420699999999998</v>
       </c>
-      <c r="G85" s="141">
+      <c r="G85" s="112">
         <v>8.4493100000000002E-2</v>
       </c>
     </row>
@@ -7480,7 +7236,7 @@
       <c r="F86" s="37">
         <v>0.21171599999999999</v>
       </c>
-      <c r="G86" s="141">
+      <c r="G86" s="112">
         <v>5.0948300000000002E-2</v>
       </c>
     </row>
@@ -7503,7 +7259,7 @@
       <c r="F87" s="37">
         <v>0.23136799999999999</v>
       </c>
-      <c r="G87" s="141">
+      <c r="G87" s="112">
         <v>7.4430300000000005E-2</v>
       </c>
     </row>
@@ -7526,7 +7282,7 @@
       <c r="F88" s="37">
         <v>0.34229399999999999</v>
       </c>
-      <c r="G88" s="141">
+      <c r="G88" s="112">
         <v>7.7721700000000005E-2</v>
       </c>
     </row>
@@ -7549,7 +7305,7 @@
       <c r="F89" s="37">
         <v>0.328457</v>
       </c>
-      <c r="G89" s="141">
+      <c r="G89" s="112">
         <v>7.3749300000000004E-2</v>
       </c>
     </row>
@@ -7572,7 +7328,7 @@
       <c r="F90" s="37">
         <v>0.33388400000000001</v>
       </c>
-      <c r="G90" s="141">
+      <c r="G90" s="112">
         <v>6.9205000000000003E-2</v>
       </c>
     </row>
@@ -7595,7 +7351,7 @@
       <c r="F91" s="37">
         <v>0.44470500000000002</v>
       </c>
-      <c r="G91" s="141">
+      <c r="G91" s="112">
         <v>8.9530799999999994E-2</v>
       </c>
     </row>
@@ -7618,7 +7374,7 @@
       <c r="F92" s="37">
         <v>0.18859999999999999</v>
       </c>
-      <c r="G92" s="141">
+      <c r="G92" s="112">
         <v>5.1705500000000001E-2</v>
       </c>
     </row>
@@ -7641,7 +7397,7 @@
       <c r="F93" s="37">
         <v>0.37837399999999999</v>
       </c>
-      <c r="G93" s="141">
+      <c r="G93" s="112">
         <v>9.5171599999999995E-2</v>
       </c>
     </row>
@@ -7664,7 +7420,7 @@
       <c r="F94" s="37">
         <v>0.459372</v>
       </c>
-      <c r="G94" s="141">
+      <c r="G94" s="112">
         <v>9.7981299999999993E-2</v>
       </c>
     </row>
@@ -7687,7 +7443,7 @@
       <c r="F95" s="37">
         <v>0.409022</v>
       </c>
-      <c r="G95" s="141">
+      <c r="G95" s="112">
         <v>8.4034999999999999E-2</v>
       </c>
     </row>
@@ -7710,7 +7466,7 @@
       <c r="F96" s="37">
         <v>0.258108</v>
       </c>
-      <c r="G96" s="141">
+      <c r="G96" s="112">
         <v>6.1423999999999999E-2</v>
       </c>
     </row>
@@ -7733,7 +7489,7 @@
       <c r="F97" s="37">
         <v>0.44827699999999998</v>
       </c>
-      <c r="G97" s="141">
+      <c r="G97" s="112">
         <v>8.4727499999999997E-2</v>
       </c>
     </row>
@@ -7756,7 +7512,7 @@
       <c r="F98" s="37">
         <v>0.380859</v>
       </c>
-      <c r="G98" s="141">
+      <c r="G98" s="112">
         <v>7.9699599999999995E-2</v>
       </c>
     </row>
@@ -7779,7 +7535,7 @@
       <c r="F99" s="37">
         <v>0.179396</v>
       </c>
-      <c r="G99" s="141">
+      <c r="G99" s="112">
         <v>4.7875099999999997E-2</v>
       </c>
     </row>
@@ -7802,7 +7558,7 @@
       <c r="F100" s="37">
         <v>0.386212</v>
       </c>
-      <c r="G100" s="141">
+      <c r="G100" s="112">
         <v>8.4019499999999997E-2</v>
       </c>
     </row>
@@ -7825,7 +7581,7 @@
       <c r="F101" s="37">
         <v>0.32669700000000002</v>
       </c>
-      <c r="G101" s="141">
+      <c r="G101" s="112">
         <v>8.8852399999999998E-2</v>
       </c>
     </row>
@@ -7848,7 +7604,7 @@
       <c r="F102" s="37">
         <v>0.45461600000000002</v>
       </c>
-      <c r="G102" s="141">
+      <c r="G102" s="112">
         <v>0.15438299999999999</v>
       </c>
     </row>
@@ -7871,7 +7627,7 @@
       <c r="F103" s="37">
         <v>0.20849699999999999</v>
       </c>
-      <c r="G103" s="141">
+      <c r="G103" s="112">
         <v>7.3032299999999994E-2</v>
       </c>
     </row>
@@ -7894,7 +7650,7 @@
       <c r="F104" s="37">
         <v>0.28194599999999997</v>
       </c>
-      <c r="G104" s="141">
+      <c r="G104" s="112">
         <v>7.7457600000000001E-2</v>
       </c>
     </row>
@@ -7917,7 +7673,7 @@
       <c r="F105" s="37">
         <v>0.2571</v>
       </c>
-      <c r="G105" s="141">
+      <c r="G105" s="112">
         <v>7.6537599999999997E-2</v>
       </c>
     </row>
@@ -7940,7 +7696,7 @@
       <c r="F106" s="37">
         <v>0.29575499999999999</v>
       </c>
-      <c r="G106" s="141">
+      <c r="G106" s="112">
         <v>7.5998399999999994E-2</v>
       </c>
     </row>
@@ -7963,7 +7719,7 @@
       <c r="F107" s="37">
         <v>0.310892</v>
       </c>
-      <c r="G107" s="141">
+      <c r="G107" s="112">
         <v>7.6906100000000005E-2</v>
       </c>
     </row>
@@ -7986,7 +7742,7 @@
       <c r="F108" s="37">
         <v>0.43532500000000002</v>
       </c>
-      <c r="G108" s="141">
+      <c r="G108" s="112">
         <v>8.5073599999999999E-2</v>
       </c>
     </row>
@@ -8009,7 +7765,7 @@
       <c r="F109" s="37">
         <v>0.46051599999999998</v>
       </c>
-      <c r="G109" s="141">
+      <c r="G109" s="112">
         <v>9.7773799999999994E-2</v>
       </c>
     </row>
@@ -8032,7 +7788,7 @@
       <c r="F110" s="37">
         <v>0.37851400000000002</v>
       </c>
-      <c r="G110" s="141">
+      <c r="G110" s="112">
         <v>0.107513</v>
       </c>
     </row>
@@ -8055,7 +7811,7 @@
       <c r="F111" s="37">
         <v>0.38189000000000001</v>
       </c>
-      <c r="G111" s="141">
+      <c r="G111" s="112">
         <v>9.9818900000000002E-2</v>
       </c>
     </row>
@@ -8078,7 +7834,7 @@
       <c r="F112" s="37">
         <v>0.44205800000000001</v>
       </c>
-      <c r="G112" s="141">
+      <c r="G112" s="112">
         <v>9.9856100000000003E-2</v>
       </c>
     </row>
@@ -8101,7 +7857,7 @@
       <c r="F113" s="37">
         <v>0.44906299999999999</v>
       </c>
-      <c r="G113" s="141">
+      <c r="G113" s="112">
         <v>8.9386699999999999E-2</v>
       </c>
     </row>
@@ -8124,7 +7880,7 @@
       <c r="F114" s="37">
         <v>0.29396899999999998</v>
       </c>
-      <c r="G114" s="141">
+      <c r="G114" s="112">
         <v>6.61577E-2</v>
       </c>
     </row>
@@ -8147,7 +7903,7 @@
       <c r="F115" s="37">
         <v>0.36777599999999999</v>
       </c>
-      <c r="G115" s="141">
+      <c r="G115" s="112">
         <v>7.3182899999999995E-2</v>
       </c>
     </row>
@@ -8170,7 +7926,7 @@
       <c r="F116" s="37">
         <v>0.380859</v>
       </c>
-      <c r="G116" s="141">
+      <c r="G116" s="112">
         <v>7.9699599999999995E-2</v>
       </c>
     </row>
@@ -8193,7 +7949,7 @@
       <c r="F117" s="37">
         <v>0.18341299999999999</v>
       </c>
-      <c r="G117" s="141">
+      <c r="G117" s="112">
         <v>5.1520099999999999E-2</v>
       </c>
     </row>
@@ -8216,7 +7972,7 @@
       <c r="F118" s="37">
         <v>0.38918999999999998</v>
       </c>
-      <c r="G118" s="141">
+      <c r="G118" s="112">
         <v>8.0030699999999996E-2</v>
       </c>
     </row>
@@ -8239,7 +7995,7 @@
       <c r="F119" s="37">
         <v>0.37492999999999999</v>
       </c>
-      <c r="G119" s="141">
+      <c r="G119" s="112">
         <v>0.100217</v>
       </c>
     </row>
@@ -8262,7 +8018,7 @@
       <c r="F120" s="37">
         <v>0.31156699999999998</v>
       </c>
-      <c r="G120" s="141">
+      <c r="G120" s="112">
         <v>0.10693999999999999</v>
       </c>
     </row>
@@ -8285,7 +8041,7 @@
       <c r="F121" s="37">
         <v>0.230654</v>
       </c>
-      <c r="G121" s="141">
+      <c r="G121" s="112">
         <v>7.7063900000000005E-2</v>
       </c>
     </row>
@@ -8308,7 +8064,7 @@
       <c r="F122" s="37">
         <v>0.27549600000000002</v>
       </c>
-      <c r="G122" s="141">
+      <c r="G122" s="112">
         <v>7.1046899999999996E-2</v>
       </c>
     </row>
@@ -8331,7 +8087,7 @@
       <c r="F123" s="37">
         <v>0.180475</v>
       </c>
-      <c r="G123" s="141">
+      <c r="G123" s="112">
         <v>5.4836299999999998E-2</v>
       </c>
     </row>
@@ -8354,7 +8110,7 @@
       <c r="F124" s="37">
         <v>0.42054999999999998</v>
       </c>
-      <c r="G124" s="141">
+      <c r="G124" s="112">
         <v>0.10097399999999999</v>
       </c>
     </row>
@@ -8377,7 +8133,7 @@
       <c r="F125" s="37">
         <v>0.40851799999999999</v>
       </c>
-      <c r="G125" s="141">
+      <c r="G125" s="112">
         <v>9.5214099999999996E-2</v>
       </c>
     </row>
@@ -8400,7 +8156,7 @@
       <c r="F126" s="37">
         <v>0.40667599999999998</v>
       </c>
-      <c r="G126" s="141">
+      <c r="G126" s="112">
         <v>8.2854800000000006E-2</v>
       </c>
     </row>
@@ -8423,7 +8179,7 @@
       <c r="F127" s="37">
         <v>0.495338</v>
       </c>
-      <c r="G127" s="141">
+      <c r="G127" s="112">
         <v>0.101115</v>
       </c>
     </row>
@@ -8446,7 +8202,7 @@
       <c r="F128" s="37">
         <v>0.52360899999999999</v>
       </c>
-      <c r="G128" s="141">
+      <c r="G128" s="112">
         <v>0.147318</v>
       </c>
     </row>
@@ -8469,7 +8225,7 @@
       <c r="F129" s="37">
         <v>0.45449699999999998</v>
       </c>
-      <c r="G129" s="141">
+      <c r="G129" s="112">
         <v>0.119767</v>
       </c>
     </row>
@@ -8492,7 +8248,7 @@
       <c r="F130" s="37">
         <v>0.40343299999999999</v>
       </c>
-      <c r="G130" s="141">
+      <c r="G130" s="112">
         <v>9.4635200000000003E-2</v>
       </c>
     </row>
@@ -8515,7 +8271,7 @@
       <c r="F131" s="37">
         <v>0.53664000000000001</v>
       </c>
-      <c r="G131" s="141">
+      <c r="G131" s="112">
         <v>0.106142</v>
       </c>
     </row>
@@ -8538,7 +8294,7 @@
       <c r="F132" s="37">
         <v>0.218719</v>
       </c>
-      <c r="G132" s="141">
+      <c r="G132" s="112">
         <v>5.20276E-2</v>
       </c>
     </row>
@@ -8561,7 +8317,7 @@
       <c r="F133" s="37">
         <v>0.355244</v>
       </c>
-      <c r="G133" s="141">
+      <c r="G133" s="112">
         <v>7.4700000000000003E-2</v>
       </c>
     </row>
@@ -8584,7 +8340,7 @@
       <c r="F134" s="37">
         <v>0.37267099999999997</v>
       </c>
-      <c r="G134" s="141">
+      <c r="G134" s="112">
         <v>7.7942899999999996E-2</v>
       </c>
     </row>
@@ -8607,7 +8363,7 @@
       <c r="F135" s="37">
         <v>0.264567</v>
       </c>
-      <c r="G135" s="141">
+      <c r="G135" s="112">
         <v>8.0192100000000002E-2</v>
       </c>
     </row>
@@ -8630,7 +8386,7 @@
       <c r="F136" s="37">
         <v>0.47795700000000002</v>
       </c>
-      <c r="G136" s="141">
+      <c r="G136" s="112">
         <v>9.3003100000000005E-2</v>
       </c>
     </row>
@@ -8653,7 +8409,7 @@
       <c r="F137" s="37">
         <v>0.51614400000000005</v>
       </c>
-      <c r="G137" s="141">
+      <c r="G137" s="112">
         <v>0.14021400000000001</v>
       </c>
     </row>
@@ -8676,7 +8432,7 @@
       <c r="F138" s="37">
         <v>0.61609199999999997</v>
       </c>
-      <c r="G138" s="141">
+      <c r="G138" s="112">
         <v>0.202345</v>
       </c>
     </row>
@@ -8699,7 +8455,7 @@
       <c r="F139" s="37">
         <v>0.26639000000000002</v>
       </c>
-      <c r="G139" s="141">
+      <c r="G139" s="112">
         <v>8.19878E-2</v>
       </c>
     </row>
@@ -8722,7 +8478,7 @@
       <c r="F140" s="37">
         <v>0.24405299999999999</v>
       </c>
-      <c r="G140" s="141">
+      <c r="G140" s="112">
         <v>5.8651200000000001E-2</v>
       </c>
     </row>
@@ -8745,7 +8501,7 @@
       <c r="F141" s="37">
         <v>0.163774</v>
       </c>
-      <c r="G141" s="141">
+      <c r="G141" s="112">
         <v>5.2653600000000002E-2</v>
       </c>
     </row>
@@ -8768,7 +8524,7 @@
       <c r="F142" s="37">
         <v>0.41799900000000001</v>
       </c>
-      <c r="G142" s="141">
+      <c r="G142" s="112">
         <v>9.4883999999999996E-2</v>
       </c>
     </row>
@@ -8791,7 +8547,7 @@
       <c r="F143" s="37">
         <v>0.32311099999999998</v>
       </c>
-      <c r="G143" s="141">
+      <c r="G143" s="112">
         <v>7.2502700000000003E-2</v>
       </c>
     </row>
@@ -8814,7 +8570,7 @@
       <c r="F144" s="37">
         <v>0.375027</v>
       </c>
-      <c r="G144" s="141">
+      <c r="G144" s="112">
         <v>7.7646499999999993E-2</v>
       </c>
     </row>
@@ -8837,7 +8593,7 @@
       <c r="F145" s="37">
         <v>0.52081699999999997</v>
       </c>
-      <c r="G145" s="141">
+      <c r="G145" s="112">
         <v>0.104738</v>
       </c>
     </row>
@@ -8860,7 +8616,7 @@
       <c r="F146" s="37">
         <v>0.38656600000000002</v>
       </c>
-      <c r="G146" s="141">
+      <c r="G146" s="112">
         <v>0.10890900000000001</v>
       </c>
     </row>
@@ -8883,7 +8639,7 @@
       <c r="F147" s="37">
         <v>0.48407099999999997</v>
       </c>
-      <c r="G147" s="141">
+      <c r="G147" s="112">
         <v>0.127695</v>
       </c>
     </row>
@@ -8906,7 +8662,7 @@
       <c r="F148" s="37">
         <v>0.54380600000000001</v>
       </c>
-      <c r="G148" s="141">
+      <c r="G148" s="112">
         <v>0.12779199999999999</v>
       </c>
     </row>
@@ -8929,7 +8685,7 @@
       <c r="F149" s="37">
         <v>0.47246100000000002</v>
       </c>
-      <c r="G149" s="141">
+      <c r="G149" s="112">
         <v>9.3412599999999998E-2</v>
       </c>
     </row>
@@ -8952,7 +8708,7 @@
       <c r="F150" s="37">
         <v>0.38531199999999999</v>
       </c>
-      <c r="G150" s="141">
+      <c r="G150" s="112">
         <v>9.1877600000000004E-2</v>
       </c>
     </row>
@@ -8975,7 +8731,7 @@
       <c r="F151" s="37">
         <v>1.47159</v>
       </c>
-      <c r="G151" s="141">
+      <c r="G151" s="112">
         <v>0.31046400000000002</v>
       </c>
     </row>
@@ -8998,7 +8754,7 @@
       <c r="F152" s="37">
         <v>0.81003099999999995</v>
       </c>
-      <c r="G152" s="141">
+      <c r="G152" s="112">
         <v>0.169795</v>
       </c>
     </row>
@@ -9021,7 +8777,7 @@
       <c r="F153" s="37">
         <v>0.204627</v>
       </c>
-      <c r="G153" s="141">
+      <c r="G153" s="112">
         <v>6.2046299999999999E-2</v>
       </c>
     </row>
@@ -9044,7 +8800,7 @@
       <c r="F154" s="37">
         <v>1.2650600000000001</v>
       </c>
-      <c r="G154" s="141">
+      <c r="G154" s="112">
         <v>0.246172</v>
       </c>
     </row>
@@ -9067,7 +8823,7 @@
       <c r="F155" s="37">
         <v>0.37946099999999999</v>
       </c>
-      <c r="G155" s="141">
+      <c r="G155" s="112">
         <v>0.10304000000000001</v>
       </c>
     </row>
@@ -9090,7 +8846,7 @@
       <c r="F156" s="37">
         <v>0.21701799999999999</v>
       </c>
-      <c r="G156" s="141">
+      <c r="G156" s="112">
         <v>7.1269700000000005E-2</v>
       </c>
     </row>
@@ -9113,7 +8869,7 @@
       <c r="F157" s="37">
         <v>0.22855900000000001</v>
       </c>
-      <c r="G157" s="141">
+      <c r="G157" s="112">
         <v>7.0344799999999999E-2</v>
       </c>
     </row>
@@ -9136,7 +8892,7 @@
       <c r="F158" s="37">
         <v>0.228106</v>
       </c>
-      <c r="G158" s="141">
+      <c r="G158" s="112">
         <v>5.4853300000000001E-2</v>
       </c>
     </row>
@@ -9159,7 +8915,7 @@
       <c r="F159" s="37">
         <v>0.24538699999999999</v>
       </c>
-      <c r="G159" s="141">
+      <c r="G159" s="112">
         <v>7.8953300000000004E-2</v>
       </c>
     </row>
@@ -9182,7 +8938,7 @@
       <c r="F160" s="37">
         <v>0.716615</v>
       </c>
-      <c r="G160" s="141">
+      <c r="G160" s="112">
         <v>0.16242100000000001</v>
       </c>
     </row>
@@ -9205,7 +8961,7 @@
       <c r="F161" s="37">
         <v>0.38388800000000001</v>
       </c>
-      <c r="G161" s="141">
+      <c r="G161" s="112">
         <v>8.6132899999999998E-2</v>
       </c>
     </row>
@@ -9228,7 +8984,7 @@
       <c r="F162" s="37">
         <v>1.05867</v>
       </c>
-      <c r="G162" s="141">
+      <c r="G162" s="112">
         <v>0.22051299999999999</v>
       </c>
     </row>
@@ -9251,7 +9007,7 @@
       <c r="F163" s="37">
         <v>0.47212599999999999</v>
       </c>
-      <c r="G163" s="141">
+      <c r="G163" s="112">
         <v>9.48576E-2</v>
       </c>
     </row>
@@ -9274,7 +9030,7 @@
       <c r="F164" s="37">
         <v>0.32430599999999998</v>
       </c>
-      <c r="G164" s="141">
+      <c r="G164" s="112">
         <v>9.8802500000000001E-2</v>
       </c>
     </row>
@@ -9297,7 +9053,7 @@
       <c r="F165" s="37">
         <v>0.35386699999999999</v>
       </c>
-      <c r="G165" s="141">
+      <c r="G165" s="112">
         <v>9.9645899999999996E-2</v>
       </c>
     </row>
@@ -9320,7 +9076,7 @@
       <c r="F166" s="37">
         <v>0.34923700000000002</v>
       </c>
-      <c r="G166" s="141">
+      <c r="G166" s="112">
         <v>8.7392399999999995E-2</v>
       </c>
     </row>
@@ -9343,7 +9099,7 @@
       <c r="F167" s="37">
         <v>0.47246100000000002</v>
       </c>
-      <c r="G167" s="141">
+      <c r="G167" s="112">
         <v>9.3412599999999998E-2</v>
       </c>
     </row>
@@ -9366,7 +9122,7 @@
       <c r="F168" s="37">
         <v>0.23527000000000001</v>
       </c>
-      <c r="G168" s="141">
+      <c r="G168" s="112">
         <v>5.8520999999999997E-2</v>
       </c>
     </row>
@@ -9389,7 +9145,7 @@
       <c r="F169" s="37">
         <v>0.31478899999999999</v>
       </c>
-      <c r="G169" s="141">
+      <c r="G169" s="112">
         <v>6.7531099999999997E-2</v>
       </c>
     </row>
@@ -9412,7 +9168,7 @@
       <c r="F170" s="37">
         <v>0.30069600000000002</v>
       </c>
-      <c r="G170" s="141">
+      <c r="G170" s="112">
         <v>6.3357800000000006E-2</v>
       </c>
     </row>
@@ -9435,7 +9191,7 @@
       <c r="F171" s="37">
         <v>0.167988</v>
       </c>
-      <c r="G171" s="141">
+      <c r="G171" s="112">
         <v>4.9786400000000001E-2</v>
       </c>
     </row>
@@ -9458,7 +9214,7 @@
       <c r="F172" s="37">
         <v>0.44997300000000001</v>
       </c>
-      <c r="G172" s="141">
+      <c r="G172" s="112">
         <v>8.5777199999999998E-2</v>
       </c>
     </row>
@@ -9481,7 +9237,7 @@
       <c r="F173" s="37">
         <v>0.47886200000000001</v>
       </c>
-      <c r="G173" s="141">
+      <c r="G173" s="112">
         <v>0.12086</v>
       </c>
     </row>
@@ -9504,7 +9260,7 @@
       <c r="F174" s="37">
         <v>0.31255899999999998</v>
       </c>
-      <c r="G174" s="141">
+      <c r="G174" s="112">
         <v>0.110626</v>
       </c>
     </row>
@@ -9527,7 +9283,7 @@
       <c r="F175" s="37">
         <v>0.242114</v>
       </c>
-      <c r="G175" s="141">
+      <c r="G175" s="112">
         <v>7.6394299999999998E-2</v>
       </c>
     </row>
@@ -9550,7 +9306,7 @@
       <c r="F176" s="37">
         <v>0.26510299999999998</v>
       </c>
-      <c r="G176" s="141">
+      <c r="G176" s="112">
         <v>6.3127500000000003E-2</v>
       </c>
     </row>
@@ -9573,7 +9329,7 @@
       <c r="F177" s="37">
         <v>0.18260199999999999</v>
       </c>
-      <c r="G177" s="141">
+      <c r="G177" s="112">
         <v>5.5004400000000002E-2</v>
       </c>
     </row>
@@ -9596,7 +9352,7 @@
       <c r="F178" s="37">
         <v>0.33567200000000003</v>
       </c>
-      <c r="G178" s="141">
+      <c r="G178" s="112">
         <v>7.3140200000000002E-2</v>
       </c>
     </row>
@@ -9619,7 +9375,7 @@
       <c r="F179" s="37">
         <v>0.237599</v>
       </c>
-      <c r="G179" s="141">
+      <c r="G179" s="112">
         <v>5.0320799999999999E-2</v>
       </c>
     </row>
@@ -9642,7 +9398,7 @@
       <c r="F180" s="37">
         <v>0.24665599999999999</v>
       </c>
-      <c r="G180" s="141">
+      <c r="G180" s="112">
         <v>5.4342500000000002E-2</v>
       </c>
     </row>
@@ -9665,7 +9421,7 @@
       <c r="F181" s="37">
         <v>0.364514</v>
       </c>
-      <c r="G181" s="141">
+      <c r="G181" s="112">
         <v>6.9290500000000005E-2</v>
       </c>
     </row>
@@ -9688,7 +9444,7 @@
       <c r="F182" s="37">
         <v>0.19736899999999999</v>
       </c>
-      <c r="G182" s="141">
+      <c r="G182" s="112">
         <v>5.3979199999999998E-2</v>
       </c>
     </row>
@@ -9711,7 +9467,7 @@
       <c r="F183" s="37">
         <v>0.40239999999999998</v>
       </c>
-      <c r="G183" s="141">
+      <c r="G183" s="112">
         <v>0.102562</v>
       </c>
     </row>
@@ -9734,7 +9490,7 @@
       <c r="F184" s="37">
         <v>0.373303</v>
       </c>
-      <c r="G184" s="141">
+      <c r="G184" s="112">
         <v>8.31152E-2</v>
       </c>
     </row>
@@ -9757,7 +9513,7 @@
       <c r="F185" s="37">
         <v>0.44384499999999999</v>
       </c>
-      <c r="G185" s="141">
+      <c r="G185" s="112">
         <v>9.0625700000000003E-2</v>
       </c>
     </row>
@@ -9780,7 +9536,7 @@
       <c r="F186" s="37">
         <v>0.23527000000000001</v>
       </c>
-      <c r="G186" s="141">
+      <c r="G186" s="112">
         <v>5.8520999999999997E-2</v>
       </c>
     </row>
@@ -9803,7 +9559,7 @@
       <c r="F187" s="37">
         <v>0.384272</v>
       </c>
-      <c r="G187" s="141">
+      <c r="G187" s="112">
         <v>7.7091900000000005E-2</v>
       </c>
     </row>
@@ -9826,7 +9582,7 @@
       <c r="F188" s="37">
         <v>0.36795899999999998</v>
       </c>
-      <c r="G188" s="141">
+      <c r="G188" s="112">
         <v>7.3715699999999995E-2</v>
       </c>
     </row>
@@ -9849,7 +9605,7 @@
       <c r="F189" s="37">
         <v>0.18529899999999999</v>
       </c>
-      <c r="G189" s="141">
+      <c r="G189" s="112">
         <v>5.3656599999999999E-2</v>
       </c>
     </row>
@@ -9872,7 +9628,7 @@
       <c r="F190" s="37">
         <v>0.44907000000000002</v>
       </c>
-      <c r="G190" s="141">
+      <c r="G190" s="112">
         <v>9.1503399999999999E-2</v>
       </c>
     </row>
@@ -9895,7 +9651,7 @@
       <c r="F191" s="37">
         <v>0.40045399999999998</v>
       </c>
-      <c r="G191" s="141">
+      <c r="G191" s="112">
         <v>0.111335</v>
       </c>
     </row>
@@ -9918,7 +9674,7 @@
       <c r="F192" s="37">
         <v>0.31080999999999998</v>
       </c>
-      <c r="G192" s="141">
+      <c r="G192" s="112">
         <v>0.101536</v>
       </c>
     </row>
@@ -9941,7 +9697,7 @@
       <c r="F193" s="37">
         <v>0.20591000000000001</v>
       </c>
-      <c r="G193" s="141">
+      <c r="G193" s="112">
         <v>6.5986100000000006E-2</v>
       </c>
     </row>
@@ -9964,7 +9720,7 @@
       <c r="F194" s="37">
         <v>0.21273800000000001</v>
       </c>
-      <c r="G194" s="141">
+      <c r="G194" s="112">
         <v>5.37966E-2</v>
       </c>
     </row>
@@ -9987,7 +9743,7 @@
       <c r="F195" s="37">
         <v>0.206868</v>
       </c>
-      <c r="G195" s="141">
+      <c r="G195" s="112">
         <v>6.5720299999999995E-2</v>
       </c>
     </row>
@@ -10010,7 +9766,7 @@
       <c r="F196" s="37">
         <v>0.34014499999999998</v>
       </c>
-      <c r="G196" s="141">
+      <c r="G196" s="112">
         <v>8.1698800000000002E-2</v>
       </c>
     </row>
@@ -10033,7 +9789,7 @@
       <c r="F197" s="37">
         <v>0.33842299999999997</v>
       </c>
-      <c r="G197" s="141">
+      <c r="G197" s="112">
         <v>8.0177899999999996E-2</v>
       </c>
     </row>
@@ -10056,7 +9812,7 @@
       <c r="F198" s="37">
         <v>0.383046</v>
       </c>
-      <c r="G198" s="141">
+      <c r="G198" s="112">
         <v>7.6463900000000001E-2</v>
       </c>
     </row>
@@ -10079,7 +9835,7 @@
       <c r="F199" s="37">
         <v>0.41350599999999998</v>
       </c>
-      <c r="G199" s="141">
+      <c r="G199" s="112">
         <v>8.6338499999999999E-2</v>
       </c>
     </row>
@@ -10102,7 +9858,7 @@
       <c r="F200" s="37">
         <v>0.18865100000000001</v>
       </c>
-      <c r="G200" s="141">
+      <c r="G200" s="112">
         <v>5.7477100000000003E-2</v>
       </c>
     </row>
@@ -10125,7 +9881,7 @@
       <c r="F201" s="37">
         <v>0.37706499999999998</v>
       </c>
-      <c r="G201" s="141">
+      <c r="G201" s="112">
         <v>0.10617699999999999</v>
       </c>
     </row>
@@ -10148,7 +9904,7 @@
       <c r="F202" s="37">
         <v>0.47255399999999997</v>
       </c>
-      <c r="G202" s="141">
+      <c r="G202" s="112">
         <v>0.118227</v>
       </c>
     </row>
@@ -10171,7 +9927,7 @@
       <c r="F203" s="37">
         <v>0.44384499999999999</v>
       </c>
-      <c r="G203" s="141">
+      <c r="G203" s="112">
         <v>9.0625700000000003E-2</v>
       </c>
     </row>
@@ -10194,7 +9950,7 @@
       <c r="F204" s="37">
         <v>0.28808499999999998</v>
       </c>
-      <c r="G204" s="141">
+      <c r="G204" s="112">
         <v>7.16387E-2</v>
       </c>
     </row>
@@ -10217,7 +9973,7 @@
       <c r="F205" s="37">
         <v>0.44758999999999999</v>
       </c>
-      <c r="G205" s="141">
+      <c r="G205" s="112">
         <v>9.6034400000000006E-2</v>
       </c>
     </row>
@@ -10240,7 +9996,7 @@
       <c r="F206" s="37">
         <v>0.48196299999999997</v>
       </c>
-      <c r="G206" s="141">
+      <c r="G206" s="112">
         <v>0.10152</v>
       </c>
     </row>
@@ -10263,7 +10019,7 @@
       <c r="F207" s="37">
         <v>0.29599300000000001</v>
       </c>
-      <c r="G207" s="141">
+      <c r="G207" s="112">
         <v>8.7792800000000004E-2</v>
       </c>
     </row>
@@ -10286,7 +10042,7 @@
       <c r="F208" s="37">
         <v>0.40145799999999998</v>
       </c>
-      <c r="G208" s="141">
+      <c r="G208" s="112">
         <v>7.6540499999999997E-2</v>
       </c>
     </row>
@@ -10309,7 +10065,7 @@
       <c r="F209" s="37">
         <v>0.32884799999999997</v>
       </c>
-      <c r="G209" s="141">
+      <c r="G209" s="112">
         <v>8.3027799999999999E-2</v>
       </c>
     </row>
@@ -10332,7 +10088,7 @@
       <c r="F210" s="37">
         <v>0.27263700000000002</v>
       </c>
-      <c r="G210" s="141">
+      <c r="G210" s="112">
         <v>9.6549800000000005E-2</v>
       </c>
     </row>
@@ -10355,7 +10111,7 @@
       <c r="F211" s="37">
         <v>0.389735</v>
       </c>
-      <c r="G211" s="141">
+      <c r="G211" s="112">
         <v>0.12311800000000001</v>
       </c>
     </row>
@@ -10378,7 +10134,7 @@
       <c r="F212" s="37">
         <v>0.179206</v>
       </c>
-      <c r="G212" s="141">
+      <c r="G212" s="112">
         <v>4.2684399999999997E-2</v>
       </c>
     </row>
@@ -10401,7 +10157,7 @@
       <c r="F213" s="37">
         <v>0.230881</v>
       </c>
-      <c r="G213" s="141">
+      <c r="G213" s="112">
         <v>6.9537399999999999E-2</v>
       </c>
     </row>
@@ -10424,7 +10180,7 @@
       <c r="F214" s="37">
         <v>0.37662899999999999</v>
       </c>
-      <c r="G214" s="141">
+      <c r="G214" s="112">
         <v>8.2053500000000001E-2</v>
       </c>
     </row>
@@ -10447,7 +10203,7 @@
       <c r="F215" s="37">
         <v>0.451706</v>
       </c>
-      <c r="G215" s="141">
+      <c r="G215" s="112">
         <v>9.5755999999999994E-2</v>
       </c>
     </row>
@@ -10470,7 +10226,7 @@
       <c r="F216" s="37">
         <v>0.34387499999999999</v>
       </c>
-      <c r="G216" s="141">
+      <c r="G216" s="112">
         <v>7.5786900000000004E-2</v>
       </c>
     </row>
@@ -10493,7 +10249,7 @@
       <c r="F217" s="37">
         <v>0.79732999999999998</v>
       </c>
-      <c r="G217" s="141">
+      <c r="G217" s="112">
         <v>0.15168999999999999</v>
       </c>
     </row>
@@ -10516,7 +10272,7 @@
       <c r="F218" s="37">
         <v>0.44472400000000001</v>
       </c>
-      <c r="G218" s="141">
+      <c r="G218" s="112">
         <v>0.12504399999999999</v>
       </c>
     </row>
@@ -10539,7 +10295,7 @@
       <c r="F219" s="37">
         <v>0.42122500000000002</v>
       </c>
-      <c r="G219" s="141">
+      <c r="G219" s="112">
         <v>0.110958</v>
       </c>
     </row>
@@ -10562,7 +10318,7 @@
       <c r="F220" s="37">
         <v>0.52118500000000001</v>
       </c>
-      <c r="G220" s="141">
+      <c r="G220" s="112">
         <v>0.122268</v>
       </c>
     </row>
@@ -10585,7 +10341,7 @@
       <c r="F221" s="37">
         <v>0.57407399999999997</v>
       </c>
-      <c r="G221" s="141">
+      <c r="G221" s="112">
         <v>0.113594</v>
       </c>
     </row>
@@ -10608,7 +10364,7 @@
       <c r="F222" s="37">
         <v>0.301788</v>
       </c>
-      <c r="G222" s="141">
+      <c r="G222" s="112">
         <v>7.17666E-2</v>
       </c>
     </row>
@@ -10631,7 +10387,7 @@
       <c r="F223" s="37">
         <v>0.49380499999999999</v>
       </c>
-      <c r="G223" s="141">
+      <c r="G223" s="112">
         <v>0.103851</v>
       </c>
     </row>
@@ -10654,7 +10410,7 @@
       <c r="F224" s="37">
         <v>0.50172899999999998</v>
       </c>
-      <c r="G224" s="141">
+      <c r="G224" s="112">
         <v>0.10496</v>
       </c>
     </row>
@@ -10677,7 +10433,7 @@
       <c r="F225" s="37">
         <v>0.28934799999999999</v>
       </c>
-      <c r="G225" s="141">
+      <c r="G225" s="112">
         <v>8.7746599999999994E-2</v>
       </c>
     </row>
@@ -10700,7 +10456,7 @@
       <c r="F226" s="37">
         <v>0.51152799999999998</v>
       </c>
-      <c r="G226" s="141">
+      <c r="G226" s="112">
         <v>9.9526400000000001E-2</v>
       </c>
     </row>
@@ -10723,7 +10479,7 @@
       <c r="F227" s="37">
         <v>0.39043499999999998</v>
       </c>
-      <c r="G227" s="141">
+      <c r="G227" s="112">
         <v>0.106061</v>
       </c>
     </row>
@@ -10746,7 +10502,7 @@
       <c r="F228" s="37">
         <v>0.38515700000000003</v>
       </c>
-      <c r="G228" s="141">
+      <c r="G228" s="112">
         <v>0.12640199999999999</v>
       </c>
     </row>
@@ -10769,7 +10525,7 @@
       <c r="F229" s="37">
         <v>0.22939999999999999</v>
       </c>
-      <c r="G229" s="141">
+      <c r="G229" s="112">
         <v>7.0670399999999994E-2</v>
       </c>
     </row>
@@ -10792,7 +10548,7 @@
       <c r="F230" s="37">
         <v>0.249472</v>
       </c>
-      <c r="G230" s="141">
+      <c r="G230" s="112">
         <v>6.0045899999999999E-2</v>
       </c>
     </row>
@@ -10815,7 +10571,7 @@
       <c r="F231" s="37">
         <v>0.174374</v>
       </c>
-      <c r="G231" s="141">
+      <c r="G231" s="112">
         <v>5.6044799999999999E-2</v>
       </c>
     </row>
@@ -10838,7 +10594,7 @@
       <c r="F232" s="37">
         <v>0.48188799999999998</v>
       </c>
-      <c r="G232" s="141">
+      <c r="G232" s="112">
         <v>0.10938199999999999</v>
       </c>
     </row>
@@ -10861,7 +10617,7 @@
       <c r="F233" s="37">
         <v>0.27595399999999998</v>
       </c>
-      <c r="G233" s="141">
+      <c r="G233" s="112">
         <v>6.1940599999999998E-2</v>
       </c>
     </row>
@@ -10884,7 +10640,7 @@
       <c r="F234" s="37">
         <v>0.43242900000000001</v>
       </c>
-      <c r="G234" s="141">
+      <c r="G234" s="112">
         <v>8.9546899999999999E-2</v>
       </c>
     </row>
@@ -10907,7 +10663,7 @@
       <c r="F235" s="37">
         <v>0.59375999999999995</v>
       </c>
-      <c r="G235" s="141">
+      <c r="G235" s="112">
         <v>0.119522</v>
       </c>
     </row>
@@ -36766,6 +36522,15 @@
       <c r="D1358" s="33" t="s">
         <v>14</v>
       </c>
+      <c r="E1358" s="38">
+        <v>1344</v>
+      </c>
+      <c r="F1358" s="32">
+        <v>0.32790999999999998</v>
+      </c>
+      <c r="G1358" s="33">
+        <v>9.23239E-2</v>
+      </c>
     </row>
     <row r="1359" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1359" s="38" t="s">
@@ -36780,6 +36545,15 @@
       <c r="D1359" s="33" t="s">
         <v>15</v>
       </c>
+      <c r="E1359" s="38">
+        <v>1140</v>
+      </c>
+      <c r="F1359" s="32">
+        <v>0.62430600000000003</v>
+      </c>
+      <c r="G1359" s="33">
+        <v>0.165161</v>
+      </c>
     </row>
     <row r="1360" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1360" s="38" t="s">
@@ -36794,8 +36568,17 @@
       <c r="D1360" s="33" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="1361" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1360" s="38">
+        <v>1380</v>
+      </c>
+      <c r="F1360" s="32">
+        <v>0.45979100000000001</v>
+      </c>
+      <c r="G1360" s="33">
+        <v>0.107943</v>
+      </c>
+    </row>
+    <row r="1361" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1361" s="38" t="s">
         <v>63</v>
       </c>
@@ -36808,8 +36591,17 @@
       <c r="D1361" s="33" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="1362" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1361" s="38">
+        <v>2079</v>
+      </c>
+      <c r="F1361" s="32">
+        <v>0.90539599999999998</v>
+      </c>
+      <c r="G1361" s="33">
+        <v>0.181781</v>
+      </c>
+    </row>
+    <row r="1362" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1362" s="38" t="s">
         <v>63</v>
       </c>
@@ -36822,8 +36614,17 @@
       <c r="D1362" s="33" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="1363" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1362" s="38">
+        <v>1480</v>
+      </c>
+      <c r="F1362" s="32">
+        <v>1.1129199999999999</v>
+      </c>
+      <c r="G1362" s="33">
+        <v>0.26367699999999999</v>
+      </c>
+    </row>
+    <row r="1363" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1363" s="38" t="s">
         <v>63</v>
       </c>
@@ -36836,8 +36637,17 @@
       <c r="D1363" s="33" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="1364" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1363" s="38">
+        <v>1318</v>
+      </c>
+      <c r="F1363" s="32">
+        <v>0.74116599999999999</v>
+      </c>
+      <c r="G1363" s="33">
+        <v>0.157494</v>
+      </c>
+    </row>
+    <row r="1364" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1364" s="38" t="s">
         <v>63</v>
       </c>
@@ -36850,8 +36660,17 @@
       <c r="D1364" s="33" t="s">
         <v>20</v>
       </c>
-    </row>
-    <row r="1365" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1364" s="38">
+        <v>1193</v>
+      </c>
+      <c r="F1364" s="32">
+        <v>0.40425800000000001</v>
+      </c>
+      <c r="G1364" s="33">
+        <v>8.5261799999999999E-2</v>
+      </c>
+    </row>
+    <row r="1365" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1365" s="38" t="s">
         <v>63</v>
       </c>
@@ -36864,8 +36683,17 @@
       <c r="D1365" s="33" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="1366" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1365" s="38">
+        <v>1966</v>
+      </c>
+      <c r="F1365" s="32">
+        <v>0.17164699999999999</v>
+      </c>
+      <c r="G1365" s="33">
+        <v>5.2616499999999997E-2</v>
+      </c>
+    </row>
+    <row r="1366" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1366" s="38" t="s">
         <v>63</v>
       </c>
@@ -36878,8 +36706,17 @@
       <c r="D1366" s="33" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="1367" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1366" s="38">
+        <v>1794</v>
+      </c>
+      <c r="F1366" s="32">
+        <v>1.1497299999999999</v>
+      </c>
+      <c r="G1366" s="33">
+        <v>0.22609799999999999</v>
+      </c>
+    </row>
+    <row r="1367" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1367" s="38" t="s">
         <v>63</v>
       </c>
@@ -36892,8 +36729,17 @@
       <c r="D1367" s="33" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="1368" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1367" s="38">
+        <v>1844</v>
+      </c>
+      <c r="F1367" s="32">
+        <v>0.26942199999999999</v>
+      </c>
+      <c r="G1367" s="33">
+        <v>7.3457400000000006E-2</v>
+      </c>
+    </row>
+    <row r="1368" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1368" s="38" t="s">
         <v>63</v>
       </c>
@@ -36906,8 +36752,17 @@
       <c r="D1368" s="33" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="1369" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1368" s="38">
+        <v>1034</v>
+      </c>
+      <c r="F1368" s="32">
+        <v>1.04921</v>
+      </c>
+      <c r="G1368" s="33">
+        <v>0.345105</v>
+      </c>
+    </row>
+    <row r="1369" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1369" s="38" t="s">
         <v>63</v>
       </c>
@@ -36920,8 +36775,17 @@
       <c r="D1369" s="33" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="1370" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1369" s="38">
+        <v>1349</v>
+      </c>
+      <c r="F1369" s="32">
+        <v>0.43065300000000001</v>
+      </c>
+      <c r="G1369" s="33">
+        <v>0.135578</v>
+      </c>
+    </row>
+    <row r="1370" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1370" s="38" t="s">
         <v>63</v>
       </c>
@@ -36934,8 +36798,17 @@
       <c r="D1370" s="33" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="1371" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1370" s="38">
+        <v>1613</v>
+      </c>
+      <c r="F1370" s="32">
+        <v>2.3339400000000001</v>
+      </c>
+      <c r="G1370" s="33">
+        <v>0.57970500000000003</v>
+      </c>
+    </row>
+    <row r="1371" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1371" s="38" t="s">
         <v>63</v>
       </c>
@@ -36948,8 +36821,17 @@
       <c r="D1371" s="33" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="1372" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1371" s="38">
+        <v>1208</v>
+      </c>
+      <c r="F1371" s="32">
+        <v>0.25817299999999999</v>
+      </c>
+      <c r="G1371" s="33">
+        <v>8.3771499999999999E-2</v>
+      </c>
+    </row>
+    <row r="1372" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1372" s="38" t="s">
         <v>63</v>
       </c>
@@ -36962,8 +36844,17 @@
       <c r="D1372" s="33" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="1373" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1372" s="38">
+        <v>1321</v>
+      </c>
+      <c r="F1372" s="32">
+        <v>0.36758000000000002</v>
+      </c>
+      <c r="G1372" s="33">
+        <v>8.4314100000000003E-2</v>
+      </c>
+    </row>
+    <row r="1373" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1373" s="38" t="s">
         <v>63</v>
       </c>
@@ -36976,8 +36867,17 @@
       <c r="D1373" s="33" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="1374" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1373" s="38">
+        <v>1299</v>
+      </c>
+      <c r="F1373" s="32">
+        <v>0.48785800000000001</v>
+      </c>
+      <c r="G1373" s="33">
+        <v>0.11103</v>
+      </c>
+    </row>
+    <row r="1374" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1374" s="38" t="s">
         <v>63</v>
       </c>
@@ -36990,8 +36890,17 @@
       <c r="D1374" s="33" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="1375" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1374" s="38">
+        <v>1008</v>
+      </c>
+      <c r="F1374" s="32">
+        <v>0.68110899999999996</v>
+      </c>
+      <c r="G1374" s="33">
+        <v>0.14157400000000001</v>
+      </c>
+    </row>
+    <row r="1375" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1375" s="38" t="s">
         <v>63</v>
       </c>
@@ -37004,10 +36913,19 @@
       <c r="D1375" s="33" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="1376" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1375" s="38">
+        <v>1106</v>
+      </c>
+      <c r="F1375" s="32">
+        <v>1.7775000000000001</v>
+      </c>
+      <c r="G1375" s="33">
+        <v>0.364618</v>
+      </c>
+    </row>
+    <row r="1376" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B1376" s="45" t="str">
-        <f t="shared" ref="B1320:B1383" si="4">IF($A1376="Daily", "n/a", "")</f>
+        <f t="shared" ref="B1376:B1383" si="4">IF($A1376="Daily", "n/a", "")</f>
         <v/>
       </c>
     </row>
@@ -47542,27 +47460,27 @@
       <c r="J1" s="84" t="s">
         <v>217</v>
       </c>
-      <c r="K1" s="129" t="s">
+      <c r="K1" s="152" t="s">
         <v>111</v>
       </c>
-      <c r="L1" s="129"/>
-      <c r="M1" s="128" t="s">
+      <c r="L1" s="152"/>
+      <c r="M1" s="151" t="s">
         <v>118</v>
       </c>
-      <c r="N1" s="128"/>
-      <c r="O1" s="128"/>
-      <c r="P1" s="128"/>
-      <c r="Q1" s="128"/>
-      <c r="R1" s="128"/>
-      <c r="S1" s="128"/>
-      <c r="T1" s="128"/>
-      <c r="U1" s="128"/>
-      <c r="V1" s="128"/>
-      <c r="W1" s="128"/>
-      <c r="X1" s="128"/>
-      <c r="Y1" s="128"/>
-      <c r="Z1" s="128"/>
-      <c r="AA1" s="128"/>
+      <c r="N1" s="151"/>
+      <c r="O1" s="151"/>
+      <c r="P1" s="151"/>
+      <c r="Q1" s="151"/>
+      <c r="R1" s="151"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="151"/>
+      <c r="U1" s="151"/>
+      <c r="V1" s="151"/>
+      <c r="W1" s="151"/>
+      <c r="X1" s="151"/>
+      <c r="Y1" s="151"/>
+      <c r="Z1" s="151"/>
+      <c r="AA1" s="151"/>
     </row>
     <row r="2" spans="1:27" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="str" cm="1">
@@ -54614,8 +54532,8 @@
   <cols>
     <col min="1" max="1" width="10.77734375" style="20" customWidth="1"/>
     <col min="2" max="2" width="15.77734375" style="45" customWidth="1"/>
-    <col min="3" max="3" width="15.77734375" style="151" customWidth="1"/>
-    <col min="4" max="4" width="15.77734375" style="153" customWidth="1"/>
+    <col min="3" max="3" width="15.77734375" style="121" customWidth="1"/>
+    <col min="4" max="4" width="15.77734375" style="123" customWidth="1"/>
     <col min="5" max="5" width="15" style="20" customWidth="1"/>
     <col min="6" max="6" width="18.77734375" style="25" customWidth="1"/>
     <col min="7" max="8" width="18.77734375" style="24" hidden="1" customWidth="1"/>
@@ -54624,72 +54542,72 @@
     <col min="14" max="16" width="15" style="20" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" s="142" customFormat="1" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="144" t="s">
+    <row r="1" spans="1:31" s="113" customFormat="1" ht="40.049999999999997" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="114" t="s">
         <v>61</v>
       </c>
-      <c r="B1" s="145" t="s">
+      <c r="B1" s="115" t="s">
         <v>188</v>
       </c>
-      <c r="C1" s="146" t="s">
+      <c r="C1" s="116" t="s">
         <v>31</v>
       </c>
-      <c r="D1" s="152" t="s">
+      <c r="D1" s="122" t="s">
         <v>166</v>
       </c>
-      <c r="E1" s="147" t="s">
+      <c r="E1" s="117" t="s">
         <v>172</v>
       </c>
-      <c r="F1" s="148" t="s">
+      <c r="F1" s="118" t="s">
         <v>168</v>
       </c>
-      <c r="G1" s="147" t="s">
+      <c r="G1" s="117" t="s">
         <v>173</v>
       </c>
-      <c r="H1" s="147" t="s">
+      <c r="H1" s="117" t="s">
         <v>174</v>
       </c>
-      <c r="I1" s="149" t="s">
+      <c r="I1" s="119" t="s">
         <v>171</v>
       </c>
-      <c r="J1" s="149" t="s">
+      <c r="J1" s="119" t="s">
         <v>175</v>
       </c>
-      <c r="K1" s="149" t="s">
+      <c r="K1" s="119" t="s">
         <v>119</v>
       </c>
-      <c r="L1" s="149" t="s">
+      <c r="L1" s="119" t="s">
         <v>120</v>
       </c>
-      <c r="M1" s="149" t="s">
+      <c r="M1" s="119" t="s">
         <v>121</v>
       </c>
-      <c r="N1" s="149" t="s">
+      <c r="N1" s="119" t="s">
         <v>122</v>
       </c>
-      <c r="O1" s="149" t="s">
+      <c r="O1" s="119" t="s">
         <v>123</v>
       </c>
-      <c r="P1" s="149" t="s">
+      <c r="P1" s="119" t="s">
         <v>124</v>
       </c>
-      <c r="Q1" s="143" t="s">
+      <c r="Q1" s="153" t="s">
         <v>118</v>
       </c>
-      <c r="R1" s="128"/>
-      <c r="S1" s="128"/>
-      <c r="T1" s="128"/>
-      <c r="U1" s="128"/>
-      <c r="V1" s="128"/>
-      <c r="W1" s="128"/>
-      <c r="X1" s="128"/>
-      <c r="Y1" s="128"/>
-      <c r="Z1" s="128"/>
-      <c r="AA1" s="128"/>
-      <c r="AB1" s="128"/>
-      <c r="AC1" s="128"/>
-      <c r="AD1" s="128"/>
-      <c r="AE1" s="128"/>
+      <c r="R1" s="151"/>
+      <c r="S1" s="151"/>
+      <c r="T1" s="151"/>
+      <c r="U1" s="151"/>
+      <c r="V1" s="151"/>
+      <c r="W1" s="151"/>
+      <c r="X1" s="151"/>
+      <c r="Y1" s="151"/>
+      <c r="Z1" s="151"/>
+      <c r="AA1" s="151"/>
+      <c r="AB1" s="151"/>
+      <c r="AC1" s="151"/>
+      <c r="AD1" s="151"/>
+      <c r="AE1" s="151"/>
     </row>
     <row r="2" spans="1:31" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42" t="str" cm="1">
@@ -54699,7 +54617,7 @@
       <c r="B2" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C2" s="150">
+      <c r="C2" s="120">
         <v>46228</v>
       </c>
       <c r="D2" s="17">
@@ -54741,7 +54659,7 @@
       <c r="B3" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C3" s="150">
+      <c r="C3" s="120">
         <v>46230</v>
       </c>
       <c r="D3" s="17">
@@ -54783,7 +54701,7 @@
       <c r="B4" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C4" s="150">
+      <c r="C4" s="120">
         <v>46231</v>
       </c>
       <c r="D4" s="17">
@@ -54825,7 +54743,7 @@
       <c r="B5" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C5" s="150">
+      <c r="C5" s="120">
         <v>46232</v>
       </c>
       <c r="D5" s="17">
@@ -54867,7 +54785,7 @@
       <c r="B6" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C6" s="150">
+      <c r="C6" s="120">
         <v>46233</v>
       </c>
       <c r="D6" s="17">
@@ -54909,7 +54827,7 @@
       <c r="B7" s="74" t="str">
         <v>31/07-error1</v>
       </c>
-      <c r="C7" s="150">
+      <c r="C7" s="120">
         <v>46234</v>
       </c>
       <c r="D7" s="17">
@@ -54951,7 +54869,7 @@
       <c r="B8" s="74" t="str">
         <v>31/07-error2</v>
       </c>
-      <c r="C8" s="150">
+      <c r="C8" s="120">
         <v>46234</v>
       </c>
       <c r="D8" s="17">
@@ -54993,7 +54911,7 @@
       <c r="B9" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C9" s="150">
+      <c r="C9" s="120">
         <v>46234</v>
       </c>
       <c r="D9" s="17">
@@ -55035,7 +54953,7 @@
       <c r="B10" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C10" s="150">
+      <c r="C10" s="120">
         <v>46235</v>
       </c>
       <c r="D10" s="17">
@@ -55077,7 +54995,7 @@
       <c r="B11" s="74" t="str">
         <v>03/08-error1</v>
       </c>
-      <c r="C11" s="150">
+      <c r="C11" s="120">
         <v>46237</v>
       </c>
       <c r="D11" s="17">
@@ -55119,7 +55037,7 @@
       <c r="B12" s="74" t="str">
         <v>03/08-error2</v>
       </c>
-      <c r="C12" s="150">
+      <c r="C12" s="120">
         <v>46237</v>
       </c>
       <c r="D12" s="17">
@@ -55161,7 +55079,7 @@
       <c r="B13" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C13" s="150">
+      <c r="C13" s="120">
         <v>46237</v>
       </c>
       <c r="D13" s="17">
@@ -55203,7 +55121,7 @@
       <c r="B14" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C14" s="150">
+      <c r="C14" s="120">
         <v>46238</v>
       </c>
       <c r="D14" s="17">
@@ -55245,7 +55163,7 @@
       <c r="B15" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C15" s="150">
+      <c r="C15" s="120">
         <v>46239</v>
       </c>
       <c r="D15" s="17">
@@ -55287,7 +55205,7 @@
       <c r="B16" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C16" s="150">
+      <c r="C16" s="120">
         <v>46240</v>
       </c>
       <c r="D16" s="17">
@@ -55329,7 +55247,7 @@
       <c r="B17" s="74" t="str">
         <v>shelf-baseline</v>
       </c>
-      <c r="C17" s="150">
+      <c r="C17" s="120">
         <v>46240</v>
       </c>
       <c r="D17" s="17">
@@ -55371,7 +55289,7 @@
       <c r="B18" s="74" t="str">
         <v>shelf-trial</v>
       </c>
-      <c r="C18" s="150">
+      <c r="C18" s="120">
         <v>46240</v>
       </c>
       <c r="D18" s="17">
@@ -55413,7 +55331,7 @@
       <c r="B19" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C19" s="150">
+      <c r="C19" s="120">
         <v>46242</v>
       </c>
       <c r="D19" s="17">
@@ -55455,7 +55373,7 @@
       <c r="B20" s="74" t="str">
         <v>auto-stop-1000-base</v>
       </c>
-      <c r="C20" s="150">
+      <c r="C20" s="120">
         <v>46242</v>
       </c>
       <c r="D20" s="17">
@@ -55497,7 +55415,7 @@
       <c r="B21" s="74" t="str">
         <v>auto-stop-2000-v1</v>
       </c>
-      <c r="C21" s="150">
+      <c r="C21" s="120">
         <v>46242</v>
       </c>
       <c r="D21" s="17">
@@ -55539,7 +55457,7 @@
       <c r="B22" s="74" t="str">
         <v>auto-stop-2000-v2</v>
       </c>
-      <c r="C22" s="150">
+      <c r="C22" s="120">
         <v>46242</v>
       </c>
       <c r="D22" s="17">
@@ -55581,7 +55499,7 @@
       <c r="B23" s="74" t="str">
         <v>auto-stop-1500-v1</v>
       </c>
-      <c r="C23" s="150">
+      <c r="C23" s="120">
         <v>46242</v>
       </c>
       <c r="D23" s="17">
@@ -55623,7 +55541,7 @@
       <c r="B24" s="74" t="str">
         <v>auto-stop-1500-v2</v>
       </c>
-      <c r="C24" s="150">
+      <c r="C24" s="120">
         <v>46242</v>
       </c>
       <c r="D24" s="17">
@@ -55665,7 +55583,7 @@
       <c r="B25" s="74" t="str">
         <v>auto-stop-1000-v2</v>
       </c>
-      <c r="C25" s="150">
+      <c r="C25" s="120">
         <v>46242</v>
       </c>
       <c r="D25" s="17">
@@ -55707,7 +55625,7 @@
       <c r="B26" s="74" t="str">
         <v>auto-stop-1000-v3</v>
       </c>
-      <c r="C26" s="150">
+      <c r="C26" s="120">
         <v>46242</v>
       </c>
       <c r="D26" s="17">
@@ -55749,7 +55667,7 @@
       <c r="B27" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C27" s="150">
+      <c r="C27" s="120">
         <v>46244</v>
       </c>
       <c r="D27" s="17">
@@ -55791,7 +55709,7 @@
       <c r="B28" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C28" s="150">
+      <c r="C28" s="120">
         <v>46245</v>
       </c>
       <c r="D28" s="17">
@@ -55833,7 +55751,7 @@
       <c r="B29" s="74" t="str">
         <v>didn't-set-volume</v>
       </c>
-      <c r="C29" s="150">
+      <c r="C29" s="120">
         <v>46246</v>
       </c>
       <c r="D29" s="17">
@@ -55875,7 +55793,7 @@
       <c r="B30" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C30" s="150">
+      <c r="C30" s="120">
         <v>46246</v>
       </c>
       <c r="D30" s="17">
@@ -55917,7 +55835,7 @@
       <c r="B31" s="74" t="str">
         <v>Wand-Wave-A1</v>
       </c>
-      <c r="C31" s="150">
+      <c r="C31" s="120">
         <v>46245</v>
       </c>
       <c r="D31" s="17">
@@ -55959,7 +55877,7 @@
       <c r="B32" s="74" t="str">
         <v>Wand-Wave-A2</v>
       </c>
-      <c r="C32" s="150">
+      <c r="C32" s="120">
         <v>46245</v>
       </c>
       <c r="D32" s="17">
@@ -56001,7 +55919,7 @@
       <c r="B33" s="74" t="str">
         <v>Wand-Wave-A3</v>
       </c>
-      <c r="C33" s="150">
+      <c r="C33" s="120">
         <v>46245</v>
       </c>
       <c r="D33" s="17">
@@ -56043,7 +55961,7 @@
       <c r="B34" s="74" t="str">
         <v>Wand-Wave-A4</v>
       </c>
-      <c r="C34" s="150">
+      <c r="C34" s="120">
         <v>46246</v>
       </c>
       <c r="D34" s="17">
@@ -56085,7 +56003,7 @@
       <c r="B35" s="74" t="str">
         <v>Wand-Wave-B1</v>
       </c>
-      <c r="C35" s="150">
+      <c r="C35" s="120">
         <v>46245</v>
       </c>
       <c r="D35" s="17">
@@ -56127,7 +56045,7 @@
       <c r="B36" s="74" t="str">
         <v>Wand-Wave-B2</v>
       </c>
-      <c r="C36" s="150">
+      <c r="C36" s="120">
         <v>46245</v>
       </c>
       <c r="D36" s="17">
@@ -56169,7 +56087,7 @@
       <c r="B37" s="74" t="str">
         <v>Wand-Wave-B3</v>
       </c>
-      <c r="C37" s="150">
+      <c r="C37" s="120">
         <v>46245</v>
       </c>
       <c r="D37" s="17">
@@ -56211,7 +56129,7 @@
       <c r="B38" s="74" t="str">
         <v>Wand-Wave-B4</v>
       </c>
-      <c r="C38" s="150">
+      <c r="C38" s="120">
         <v>46246</v>
       </c>
       <c r="D38" s="17">
@@ -56253,7 +56171,7 @@
       <c r="B39" s="74" t="str">
         <v>Wand-Wave-C1</v>
       </c>
-      <c r="C39" s="150">
+      <c r="C39" s="120">
         <v>46245</v>
       </c>
       <c r="D39" s="17">
@@ -56295,7 +56213,7 @@
       <c r="B40" s="74" t="str">
         <v>Wand-Wave-C2</v>
       </c>
-      <c r="C40" s="150">
+      <c r="C40" s="120">
         <v>46245</v>
       </c>
       <c r="D40" s="17">
@@ -56337,7 +56255,7 @@
       <c r="B41" s="74" t="str">
         <v>Wand-Wave-C3</v>
       </c>
-      <c r="C41" s="150">
+      <c r="C41" s="120">
         <v>46245</v>
       </c>
       <c r="D41" s="17">
@@ -56379,7 +56297,7 @@
       <c r="B42" s="74" t="str">
         <v>Wand-Wave-C4</v>
       </c>
-      <c r="C42" s="150">
+      <c r="C42" s="120">
         <v>46246</v>
       </c>
       <c r="D42" s="17">
@@ -56421,7 +56339,7 @@
       <c r="B43" s="74" t="str">
         <v>Wand-Wave-D1</v>
       </c>
-      <c r="C43" s="150">
+      <c r="C43" s="120">
         <v>46245</v>
       </c>
       <c r="D43" s="17">
@@ -56463,7 +56381,7 @@
       <c r="B44" s="74" t="str">
         <v>Wand-Wave-D2</v>
       </c>
-      <c r="C44" s="150">
+      <c r="C44" s="120">
         <v>46245</v>
       </c>
       <c r="D44" s="17">
@@ -56505,7 +56423,7 @@
       <c r="B45" s="74" t="str">
         <v>Wand-Wave-D3</v>
       </c>
-      <c r="C45" s="150">
+      <c r="C45" s="120">
         <v>46245</v>
       </c>
       <c r="D45" s="17">
@@ -56547,7 +56465,7 @@
       <c r="B46" s="74" t="str">
         <v>Wand-Wave-D4</v>
       </c>
-      <c r="C46" s="150">
+      <c r="C46" s="120">
         <v>46246</v>
       </c>
       <c r="D46" s="17">
@@ -56589,7 +56507,7 @@
       <c r="B47" s="74" t="str">
         <v>Wand-Wave-E1</v>
       </c>
-      <c r="C47" s="150">
+      <c r="C47" s="120">
         <v>46245</v>
       </c>
       <c r="D47" s="17">
@@ -56631,7 +56549,7 @@
       <c r="B48" s="74" t="str">
         <v>Wand-Wave-E2</v>
       </c>
-      <c r="C48" s="150">
+      <c r="C48" s="120">
         <v>46245</v>
       </c>
       <c r="D48" s="17">
@@ -56673,7 +56591,7 @@
       <c r="B49" s="74" t="str">
         <v>Wand-Wave-E3</v>
       </c>
-      <c r="C49" s="150">
+      <c r="C49" s="120">
         <v>46245</v>
       </c>
       <c r="D49" s="17">
@@ -56715,7 +56633,7 @@
       <c r="B50" s="74" t="str">
         <v>Wand-Wave-E4</v>
       </c>
-      <c r="C50" s="150">
+      <c r="C50" s="120">
         <v>46246</v>
       </c>
       <c r="D50" s="17">
@@ -56757,7 +56675,7 @@
       <c r="B51" s="74" t="str">
         <v>Wand-Wave-F1</v>
       </c>
-      <c r="C51" s="150">
+      <c r="C51" s="120">
         <v>46246</v>
       </c>
       <c r="D51" s="17">
@@ -56799,7 +56717,7 @@
       <c r="B52" s="74" t="str">
         <v>Wand-Wave-F2</v>
       </c>
-      <c r="C52" s="150">
+      <c r="C52" s="120">
         <v>46246</v>
       </c>
       <c r="D52" s="17">
@@ -56841,7 +56759,7 @@
       <c r="B53" s="74" t="str">
         <v>Wand-Wave-F3</v>
       </c>
-      <c r="C53" s="150">
+      <c r="C53" s="120">
         <v>46246</v>
       </c>
       <c r="D53" s="17">
@@ -56883,7 +56801,7 @@
       <c r="B54" s="74" t="str">
         <v>Wand-Wave-F4</v>
       </c>
-      <c r="C54" s="150">
+      <c r="C54" s="120">
         <v>46246</v>
       </c>
       <c r="D54" s="17">
@@ -56925,7 +56843,7 @@
       <c r="B55" s="74" t="str">
         <v>Wand-Wave-G1</v>
       </c>
-      <c r="C55" s="150">
+      <c r="C55" s="120">
         <v>46246</v>
       </c>
       <c r="D55" s="17">
@@ -56967,7 +56885,7 @@
       <c r="B56" s="74" t="str">
         <v>Wand-Wave-G2</v>
       </c>
-      <c r="C56" s="151">
+      <c r="C56" s="121">
         <v>46246</v>
       </c>
       <c r="D56" s="17">
@@ -57009,7 +56927,7 @@
       <c r="B57" s="74" t="str">
         <v>Wand-Wave-G3</v>
       </c>
-      <c r="C57" s="151">
+      <c r="C57" s="121">
         <v>46246</v>
       </c>
       <c r="D57" s="17">
@@ -57051,7 +56969,7 @@
       <c r="B58" s="74" t="str">
         <v>Wand-Wave-G4</v>
       </c>
-      <c r="C58" s="151">
+      <c r="C58" s="121">
         <v>46246</v>
       </c>
       <c r="D58" s="17">
@@ -57093,7 +57011,7 @@
       <c r="B59" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C59" s="151">
+      <c r="C59" s="121">
         <v>46247</v>
       </c>
       <c r="D59" s="17">
@@ -57135,7 +57053,7 @@
       <c r="B60" s="74" t="str">
         <v>cannot-set-volume</v>
       </c>
-      <c r="C60" s="151">
+      <c r="C60" s="121">
         <v>46248</v>
       </c>
       <c r="D60" s="17">
@@ -57177,7 +57095,7 @@
       <c r="B61" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C61" s="151">
+      <c r="C61" s="121">
         <v>46248</v>
       </c>
       <c r="D61" s="17">
@@ -57219,7 +57137,7 @@
       <c r="B62" s="74" t="str">
         <v>pre-calibrate-1</v>
       </c>
-      <c r="C62" s="151">
+      <c r="C62" s="121">
         <v>46251</v>
       </c>
       <c r="D62" s="17">
@@ -57261,7 +57179,7 @@
       <c r="B63" s="74" t="str">
         <v>pre-calibrate-2</v>
       </c>
-      <c r="C63" s="151">
+      <c r="C63" s="121">
         <v>46251</v>
       </c>
       <c r="D63" s="17">
@@ -57303,7 +57221,7 @@
       <c r="B64" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C64" s="151">
+      <c r="C64" s="121">
         <v>46251</v>
       </c>
       <c r="D64" s="17">
@@ -57345,7 +57263,7 @@
       <c r="B65" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C65" s="151">
+      <c r="C65" s="121">
         <v>46252</v>
       </c>
       <c r="D65" s="17">
@@ -57387,7 +57305,7 @@
       <c r="B66" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C66" s="151">
+      <c r="C66" s="121">
         <v>46253</v>
       </c>
       <c r="D66" s="17">
@@ -57429,7 +57347,7 @@
       <c r="B67" s="74" t="str">
         <v>20/08-error1</v>
       </c>
-      <c r="C67" s="151">
+      <c r="C67" s="121">
         <v>46254</v>
       </c>
       <c r="D67" s="17">
@@ -57471,7 +57389,7 @@
       <c r="B68" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C68" s="151">
+      <c r="C68" s="121">
         <v>46254</v>
       </c>
       <c r="D68" s="17">
@@ -57513,7 +57431,7 @@
       <c r="B69" s="74" t="str">
         <v>speed_cam11_slow_1</v>
       </c>
-      <c r="C69" s="151">
+      <c r="C69" s="121">
         <v>46253</v>
       </c>
       <c r="D69" s="17">
@@ -57555,7 +57473,7 @@
       <c r="B70" s="74" t="str">
         <v>speed_cam11_slow_2</v>
       </c>
-      <c r="C70" s="151">
+      <c r="C70" s="121">
         <v>46253</v>
       </c>
       <c r="D70" s="17">
@@ -57597,7 +57515,7 @@
       <c r="B71" s="74" t="str">
         <v>speed_cam11_fast_1</v>
       </c>
-      <c r="C71" s="151">
+      <c r="C71" s="121">
         <v>46253</v>
       </c>
       <c r="D71" s="17">
@@ -57639,7 +57557,7 @@
       <c r="B72" s="74" t="str">
         <v>speed_cam11_fast_2</v>
       </c>
-      <c r="C72" s="151">
+      <c r="C72" s="121">
         <v>46253</v>
       </c>
       <c r="D72" s="17">
@@ -57681,7 +57599,7 @@
       <c r="B73" s="74" t="str">
         <v>speed_cam11_slow_3</v>
       </c>
-      <c r="C73" s="151">
+      <c r="C73" s="121">
         <v>46253</v>
       </c>
       <c r="D73" s="17">
@@ -57723,7 +57641,7 @@
       <c r="B74" s="74" t="str">
         <v>speed_cam11_fast_3</v>
       </c>
-      <c r="C74" s="151">
+      <c r="C74" s="121">
         <v>46253</v>
       </c>
       <c r="D74" s="17">
@@ -57765,7 +57683,7 @@
       <c r="B75" s="74" t="str">
         <v>no-reset-grayscale-all</v>
       </c>
-      <c r="C75" s="151">
+      <c r="C75" s="121">
         <v>46255</v>
       </c>
       <c r="D75" s="17">
@@ -57807,7 +57725,7 @@
       <c r="B76" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C76" s="151">
+      <c r="C76" s="121">
         <v>46255</v>
       </c>
       <c r="D76" s="17">
@@ -57849,7 +57767,7 @@
       <c r="B77" s="74" t="str">
         <v>reflection-trial-2</v>
       </c>
-      <c r="C77" s="151">
+      <c r="C77" s="121">
         <v>46255</v>
       </c>
       <c r="D77" s="17">
@@ -57891,7 +57809,7 @@
       <c r="B78" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C78" s="151">
+      <c r="C78" s="121">
         <v>46258</v>
       </c>
       <c r="D78" s="17">
@@ -57933,7 +57851,7 @@
       <c r="B79" s="74" t="str">
         <v>n/a</v>
       </c>
-      <c r="C79" s="151">
+      <c r="C79" s="121">
         <v>46260</v>
       </c>
       <c r="D79" s="17">
@@ -57975,7 +57893,7 @@
       <c r="B80" s="74" t="str">
         <v>26-08-not-relative</v>
       </c>
-      <c r="C80" s="151">
+      <c r="C80" s="121">
         <v>46260</v>
       </c>
       <c r="D80" s="17">
@@ -58017,7 +57935,7 @@
       <c r="B81" s="74" t="str">
         <v>glove-capture-1</v>
       </c>
-      <c r="C81" s="151">
+      <c r="C81" s="121">
         <v>46260</v>
       </c>
       <c r="D81" s="17">
@@ -58059,7 +57977,7 @@
       <c r="B82" s="74" t="str">
         <v>glove-capture-2</v>
       </c>
-      <c r="C82" s="151">
+      <c r="C82" s="121">
         <v>46260</v>
       </c>
       <c r="D82" s="17">
@@ -58101,36 +58019,36 @@
       <c r="B83" s="74" t="str">
         <v>glove-capture-3</v>
       </c>
-      <c r="C83" s="151">
+      <c r="C83" s="121">
         <v>46260</v>
       </c>
       <c r="D83" s="17">
         <f>Sets!$G83</f>
         <v>1000</v>
       </c>
-      <c r="E83" s="7" t="e">
+      <c r="E83" s="7">
         <f>AVERAGEIFS(Log!$E$3:$E$3000, Log!$A$3:$A$3000, $A83, Log!$B$3:$B$3000, $B83, Log!$C$3:$C$3000, $C83)</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="F83" s="18" t="e">
+        <v>1415.3333333333333</v>
+      </c>
+      <c r="F83" s="18">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
+        <v>1.4153333333333333</v>
       </c>
       <c r="G83" s="17"/>
       <c r="H83" s="17"/>
       <c r="I83" s="63"/>
       <c r="J83" s="63"/>
-      <c r="K83" s="6" t="e">
+      <c r="K83" s="6">
         <f>AVERAGEIFS(Log!$F$3:$F$3000, Log!$A$3:$A$3000, $A83, Log!$B$3:$B$3000, $B83, Log!$C$3:$C$3000, $C83)</f>
-        <v>#DIV/0!</v>
+        <v>0.75292049999999988</v>
       </c>
       <c r="L83" s="6">
         <f>_xlfn.MINIFS(Log!$F$3:$F$3000, Log!$A$3:$A$3000, $A83, Log!$B$3:$B$3000, $B83, Log!$C$3:$C$3000, $C83)</f>
-        <v>0</v>
+        <v>0.17164699999999999</v>
       </c>
       <c r="M83" s="6">
         <f>_xlfn.MAXIFS(Log!$F$3:$F$3000, Log!$A$3:$A$3000, $A83, Log!$B$3:$B$3000, $B83, Log!$C$3:$C$3000, $C83)</f>
-        <v>0</v>
+        <v>2.3339400000000001</v>
       </c>
       <c r="N83" s="6"/>
       <c r="O83" s="6"/>
@@ -58143,7 +58061,7 @@
       <c r="B84" s="74" t="str">
         <v/>
       </c>
-      <c r="C84" s="151">
+      <c r="C84" s="121">
         <v>0</v>
       </c>
       <c r="E84" s="7"/>
@@ -63066,10 +62984,10 @@
       <c r="V1" s="88"/>
     </row>
     <row r="2" spans="1:25" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="130" t="s">
+      <c r="A2" s="125" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="131"/>
+      <c r="B2" s="126"/>
       <c r="C2" s="89"/>
       <c r="D2" s="89"/>
       <c r="E2" s="89"/>
@@ -63113,60 +63031,59 @@
       <c r="B3" s="91" t="s">
         <v>220</v>
       </c>
-      <c r="C3" s="92" t="str" cm="1">
-        <f t="array" ref="C3:T3">LEFT(TRANSPOSE('[1]Data-Lists'!A4:A21), 3)</f>
-        <v xml:space="preserve">#1 </v>
-      </c>
-      <c r="D3" s="92" t="str">
-        <v xml:space="preserve">#2 </v>
-      </c>
-      <c r="E3" s="92" t="str">
-        <v xml:space="preserve">#3 </v>
-      </c>
-      <c r="F3" s="92" t="str">
-        <v xml:space="preserve">#4 </v>
-      </c>
-      <c r="G3" s="92" t="str">
-        <v xml:space="preserve">#5 </v>
-      </c>
-      <c r="H3" s="92" t="str">
-        <v xml:space="preserve">#6 </v>
-      </c>
-      <c r="I3" s="92" t="str">
-        <v xml:space="preserve">#7 </v>
-      </c>
-      <c r="J3" s="93" t="str">
-        <v xml:space="preserve">#8 </v>
-      </c>
-      <c r="K3" s="92" t="str">
-        <v xml:space="preserve">#9 </v>
-      </c>
-      <c r="L3" s="92" t="str">
-        <v>#10</v>
-      </c>
-      <c r="M3" s="92" t="str">
-        <v>#11</v>
-      </c>
-      <c r="N3" s="92" t="str">
-        <v>#12</v>
-      </c>
-      <c r="O3" s="93" t="str">
-        <v>#13</v>
-      </c>
-      <c r="P3" s="92" t="str">
-        <v>#14</v>
-      </c>
-      <c r="Q3" s="92" t="str">
-        <v>#15</v>
-      </c>
-      <c r="R3" s="92" t="str">
-        <v>#16</v>
-      </c>
-      <c r="S3" s="92" t="str">
-        <v>#17</v>
-      </c>
-      <c r="T3" s="92" t="str">
-        <v>#18</v>
+      <c r="C3" s="92" t="s">
+        <v>244</v>
+      </c>
+      <c r="D3" s="92" t="s">
+        <v>245</v>
+      </c>
+      <c r="E3" s="92" t="s">
+        <v>246</v>
+      </c>
+      <c r="F3" s="92" t="s">
+        <v>247</v>
+      </c>
+      <c r="G3" s="92" t="s">
+        <v>248</v>
+      </c>
+      <c r="H3" s="92" t="s">
+        <v>249</v>
+      </c>
+      <c r="I3" s="92" t="s">
+        <v>250</v>
+      </c>
+      <c r="J3" s="93" t="s">
+        <v>251</v>
+      </c>
+      <c r="K3" s="92" t="s">
+        <v>252</v>
+      </c>
+      <c r="L3" s="92" t="s">
+        <v>253</v>
+      </c>
+      <c r="M3" s="92" t="s">
+        <v>254</v>
+      </c>
+      <c r="N3" s="92" t="s">
+        <v>255</v>
+      </c>
+      <c r="O3" s="93" t="s">
+        <v>256</v>
+      </c>
+      <c r="P3" s="92" t="s">
+        <v>257</v>
+      </c>
+      <c r="Q3" s="92" t="s">
+        <v>258</v>
+      </c>
+      <c r="R3" s="92" t="s">
+        <v>259</v>
+      </c>
+      <c r="S3" s="92" t="s">
+        <v>260</v>
+      </c>
+      <c r="T3" s="92" t="s">
+        <v>261</v>
       </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
@@ -63191,22 +63108,22 @@
       <c r="V6" s="99" t="s">
         <v>222</v>
       </c>
-      <c r="W6" s="132" t="s">
+      <c r="W6" s="127" t="s">
         <v>223</v>
       </c>
-      <c r="X6" s="133"/>
-      <c r="Y6" s="134"/>
+      <c r="X6" s="128"/>
+      <c r="Y6" s="129"/>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" s="19">
         <v>46232</v>
       </c>
       <c r="V7" s="100"/>
-      <c r="W7" s="132" t="s">
+      <c r="W7" s="127" t="s">
         <v>243</v>
       </c>
-      <c r="X7" s="133"/>
-      <c r="Y7" s="134"/>
+      <c r="X7" s="128"/>
+      <c r="Y7" s="129"/>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" s="19">
@@ -63342,7 +63259,7 @@
       <c r="A27" s="19">
         <v>46260</v>
       </c>
-      <c r="B27" s="154" t="s">
+      <c r="B27" s="124" t="s">
         <v>242</v>
       </c>
     </row>

</xml_diff>